<commit_message>
coreccion de columnas a la hora  de cargar los datos de los estudiantes y representantes  con migragr_exel
</commit_message>
<xml_diff>
--- a/Matricula_3er_grado.xlsx
+++ b/Matricula_3er_grado.xlsx
@@ -1,25 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="5" rupBuild="14420"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="21727"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Escuela Juana R\Desktop\año escolar 2025-2026 matricula\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D15C0526-C0C7-4E43-AD03-E2FD7E3F7A8A}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="1800" windowWidth="20490" windowHeight="7530" tabRatio="278"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="278" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="152511" iterateDelta="1E-4"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
       </xcalcf:calcFeatures>
     </ext>
   </extLst>
@@ -563,7 +563,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -653,24 +653,11 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="10">
     <border>
       <left/>
       <right/>
       <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
       <bottom/>
       <diagonal/>
     </border>
@@ -738,28 +725,6 @@
         <color auto="1"/>
       </left>
       <right/>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
       <top/>
       <bottom/>
       <diagonal/>
@@ -805,7 +770,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="61">
+  <cellXfs count="47">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
@@ -817,162 +782,124 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="5" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1010,7 +937,7 @@
         <xdr:cNvPr id="2" name="Image 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -1300,15 +1227,15 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A5:AE38"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A5:AE31"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="14.25"/>
   <cols>
     <col min="1" max="1" width="9" style="2"/>
     <col min="2" max="2" width="16.7109375" style="2" customWidth="1"/>
     <col min="3" max="3" width="20" style="2" customWidth="1"/>
     <col min="4" max="4" width="16.28515625" style="2" customWidth="1"/>
-    <col min="5" max="5" width="14.42578125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="23.42578125" style="2" customWidth="1"/>
     <col min="6" max="6" width="17.140625" style="2" customWidth="1"/>
     <col min="7" max="10" width="9" style="2"/>
     <col min="11" max="11" width="10.28515625" style="2" customWidth="1"/>
@@ -1327,165 +1254,165 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:31" ht="30.95" customHeight="1">
-      <c r="A5" s="37" t="s">
+      <c r="A5" s="41" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="38"/>
-      <c r="C5" s="38"/>
-      <c r="D5" s="38"/>
-      <c r="E5" s="38"/>
-      <c r="F5" s="38"/>
-      <c r="G5" s="38"/>
-      <c r="H5" s="38"/>
-      <c r="I5" s="38"/>
-      <c r="J5" s="38"/>
-      <c r="K5" s="38"/>
-      <c r="L5" s="38"/>
-      <c r="M5" s="38"/>
-      <c r="N5" s="38"/>
-      <c r="O5" s="38"/>
-      <c r="P5" s="38"/>
-      <c r="Q5" s="38"/>
-      <c r="R5" s="38"/>
-      <c r="S5" s="38"/>
-      <c r="T5" s="38"/>
-      <c r="U5" s="38"/>
-      <c r="V5" s="38"/>
-      <c r="W5" s="31"/>
-      <c r="X5" s="31"/>
+      <c r="B5" s="42"/>
+      <c r="C5" s="42"/>
+      <c r="D5" s="42"/>
+      <c r="E5" s="42"/>
+      <c r="F5" s="42"/>
+      <c r="G5" s="42"/>
+      <c r="H5" s="42"/>
+      <c r="I5" s="42"/>
+      <c r="J5" s="42"/>
+      <c r="K5" s="42"/>
+      <c r="L5" s="42"/>
+      <c r="M5" s="42"/>
+      <c r="N5" s="42"/>
+      <c r="O5" s="42"/>
+      <c r="P5" s="42"/>
+      <c r="Q5" s="42"/>
+      <c r="R5" s="42"/>
+      <c r="S5" s="42"/>
+      <c r="T5" s="42"/>
+      <c r="U5" s="42"/>
+      <c r="V5" s="42"/>
+      <c r="W5" s="27"/>
+      <c r="X5" s="27"/>
       <c r="Y5" s="1"/>
-      <c r="Z5" s="31"/>
-      <c r="AA5" s="31"/>
-      <c r="AB5" s="31"/>
+      <c r="Z5" s="27"/>
+      <c r="AA5" s="27"/>
+      <c r="AB5" s="27"/>
       <c r="AC5" s="1"/>
-      <c r="AD5" s="31"/>
-      <c r="AE5" s="31"/>
+      <c r="AD5" s="27"/>
+      <c r="AE5" s="27"/>
     </row>
     <row r="6" spans="1:31" ht="27.95" customHeight="1">
-      <c r="A6" s="32" t="s">
+      <c r="A6" s="36" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="32"/>
-      <c r="C6" s="32" t="s">
+      <c r="B6" s="36"/>
+      <c r="C6" s="36" t="s">
         <v>151</v>
       </c>
-      <c r="D6" s="32"/>
-      <c r="E6" s="32" t="s">
+      <c r="D6" s="36"/>
+      <c r="E6" s="36" t="s">
         <v>152</v>
       </c>
-      <c r="F6" s="32"/>
-      <c r="G6" s="32"/>
-      <c r="H6" s="32"/>
-      <c r="I6" s="32" t="s">
+      <c r="F6" s="36"/>
+      <c r="G6" s="36"/>
+      <c r="H6" s="36"/>
+      <c r="I6" s="36" t="s">
         <v>153</v>
       </c>
-      <c r="J6" s="32"/>
-      <c r="K6" s="32"/>
-      <c r="L6" s="32"/>
-      <c r="M6" s="32" t="s">
+      <c r="J6" s="36"/>
+      <c r="K6" s="36"/>
+      <c r="L6" s="36"/>
+      <c r="M6" s="36" t="s">
         <v>154</v>
       </c>
-      <c r="N6" s="32"/>
-      <c r="O6" s="32"/>
-      <c r="P6" s="32"/>
-      <c r="Q6" s="32" t="s">
+      <c r="N6" s="36"/>
+      <c r="O6" s="36"/>
+      <c r="P6" s="36"/>
+      <c r="Q6" s="36" t="s">
         <v>155</v>
       </c>
-      <c r="R6" s="32"/>
-      <c r="S6" s="34" t="s">
+      <c r="R6" s="36"/>
+      <c r="S6" s="38" t="s">
         <v>156</v>
       </c>
-      <c r="T6" s="35"/>
-      <c r="U6" s="35"/>
-      <c r="V6" s="36"/>
-      <c r="W6" s="31"/>
-      <c r="X6" s="31"/>
-      <c r="Z6" s="33"/>
-      <c r="AA6" s="33"/>
-      <c r="AB6" s="33"/>
+      <c r="T6" s="39"/>
+      <c r="U6" s="39"/>
+      <c r="V6" s="40"/>
+      <c r="W6" s="27"/>
+      <c r="X6" s="27"/>
+      <c r="Z6" s="37"/>
+      <c r="AA6" s="37"/>
+      <c r="AB6" s="37"/>
       <c r="AC6" s="1"/>
-      <c r="AD6" s="33"/>
-      <c r="AE6" s="33"/>
+      <c r="AD6" s="37"/>
+      <c r="AE6" s="37"/>
     </row>
     <row r="7" spans="1:31" ht="36" customHeight="1">
-      <c r="A7" s="45" t="s">
+      <c r="A7" s="33" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="46"/>
-      <c r="C7" s="47"/>
-      <c r="D7" s="39" t="s">
+      <c r="B7" s="34"/>
+      <c r="C7" s="35"/>
+      <c r="D7" s="26" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="39"/>
-      <c r="F7" s="39" t="s">
+      <c r="E7" s="26"/>
+      <c r="F7" s="26" t="s">
         <v>0</v>
       </c>
-      <c r="G7" s="39"/>
-      <c r="H7" s="39" t="s">
+      <c r="G7" s="26"/>
+      <c r="H7" s="26" t="s">
         <v>162</v>
       </c>
-      <c r="I7" s="39"/>
-      <c r="J7" s="39"/>
-      <c r="K7" s="45" t="s">
+      <c r="I7" s="26"/>
+      <c r="J7" s="26"/>
+      <c r="K7" s="33" t="s">
         <v>161</v>
       </c>
-      <c r="L7" s="47"/>
-      <c r="M7" s="39" t="s">
+      <c r="L7" s="35"/>
+      <c r="M7" s="26" t="s">
         <v>160</v>
       </c>
-      <c r="N7" s="39"/>
-      <c r="O7" s="39" t="s">
+      <c r="N7" s="26"/>
+      <c r="O7" s="26" t="s">
         <v>159</v>
       </c>
-      <c r="P7" s="39"/>
-      <c r="Q7" s="39"/>
-      <c r="R7" s="39"/>
-      <c r="S7" s="8" t="s">
+      <c r="P7" s="26"/>
+      <c r="Q7" s="26"/>
+      <c r="R7" s="26"/>
+      <c r="S7" s="7" t="s">
         <v>158</v>
       </c>
-      <c r="T7" s="8" t="s">
+      <c r="T7" s="7" t="s">
         <v>157</v>
       </c>
-      <c r="U7" s="41" t="s">
+      <c r="U7" s="29" t="s">
         <v>165</v>
       </c>
-      <c r="V7" s="42"/>
+      <c r="V7" s="30"/>
       <c r="W7" s="3"/>
       <c r="AA7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="AB7" s="31"/>
-      <c r="AC7" s="31"/>
-      <c r="AD7" s="31"/>
+      <c r="AB7" s="27"/>
+      <c r="AC7" s="27"/>
+      <c r="AD7" s="27"/>
       <c r="AE7" s="4"/>
     </row>
     <row r="8" spans="1:31" ht="17.100000000000001" customHeight="1">
-      <c r="A8" s="40" t="s">
+      <c r="A8" s="28" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="40"/>
-      <c r="C8" s="40"/>
-      <c r="D8" s="40"/>
-      <c r="E8" s="40"/>
-      <c r="F8" s="40"/>
-      <c r="G8" s="40"/>
-      <c r="H8" s="40"/>
-      <c r="I8" s="40"/>
-      <c r="J8" s="40"/>
-      <c r="K8" s="40"/>
-      <c r="L8" s="40"/>
-      <c r="M8" s="40"/>
-      <c r="N8" s="40"/>
-      <c r="O8" s="40"/>
-      <c r="P8" s="40"/>
-      <c r="Q8" s="43" t="s">
+      <c r="B8" s="28"/>
+      <c r="C8" s="28"/>
+      <c r="D8" s="28"/>
+      <c r="E8" s="28"/>
+      <c r="F8" s="28"/>
+      <c r="G8" s="28"/>
+      <c r="H8" s="28"/>
+      <c r="I8" s="28"/>
+      <c r="J8" s="28"/>
+      <c r="K8" s="28"/>
+      <c r="L8" s="28"/>
+      <c r="M8" s="28"/>
+      <c r="N8" s="28"/>
+      <c r="O8" s="28"/>
+      <c r="P8" s="28"/>
+      <c r="Q8" s="31" t="s">
         <v>3</v>
       </c>
-      <c r="R8" s="44"/>
-      <c r="S8" s="44"/>
-      <c r="T8" s="44"/>
-      <c r="U8" s="44"/>
-      <c r="V8" s="44"/>
+      <c r="R8" s="32"/>
+      <c r="S8" s="32"/>
+      <c r="T8" s="32"/>
+      <c r="U8" s="32"/>
+      <c r="V8" s="32"/>
       <c r="W8" s="4"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
@@ -1497,1467 +1424,1444 @@
       <c r="AE8" s="4"/>
     </row>
     <row r="9" spans="1:31" ht="15">
-      <c r="A9" s="48" t="s">
+      <c r="A9" s="25" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="48" t="s">
+      <c r="B9" s="25" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="49" t="s">
+      <c r="C9" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="48" t="s">
+      <c r="D9" s="25" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="48"/>
-      <c r="F9" s="48" t="s">
+      <c r="E9" s="25"/>
+      <c r="F9" s="25" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="48" t="s">
+      <c r="G9" s="25" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="48" t="s">
+      <c r="H9" s="25" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="48"/>
-      <c r="J9" s="48"/>
-      <c r="K9" s="48" t="s">
+      <c r="I9" s="25"/>
+      <c r="J9" s="25"/>
+      <c r="K9" s="25" t="s">
         <v>10</v>
       </c>
-      <c r="L9" s="48" t="s">
+      <c r="L9" s="25" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="48"/>
-      <c r="N9" s="48" t="s">
+      <c r="M9" s="25"/>
+      <c r="N9" s="25" t="s">
         <v>22</v>
       </c>
-      <c r="O9" s="48"/>
-      <c r="P9" s="48"/>
-      <c r="Q9" s="52" t="s">
+      <c r="O9" s="25"/>
+      <c r="P9" s="25"/>
+      <c r="Q9" s="43" t="s">
         <v>12</v>
       </c>
-      <c r="R9" s="53"/>
-      <c r="S9" s="48" t="s">
+      <c r="R9" s="43"/>
+      <c r="S9" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="T9" s="48" t="s">
+      <c r="T9" s="25" t="s">
         <v>23</v>
       </c>
-      <c r="U9" s="48" t="s">
+      <c r="U9" s="25" t="s">
         <v>24</v>
       </c>
-      <c r="V9" s="51" t="s">
+      <c r="V9" s="24" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="15">
-      <c r="A10" s="48"/>
-      <c r="B10" s="48"/>
-      <c r="C10" s="50"/>
-      <c r="D10" s="48"/>
-      <c r="E10" s="48"/>
-      <c r="F10" s="48"/>
-      <c r="G10" s="48"/>
-      <c r="H10" s="5" t="s">
+      <c r="A10" s="25"/>
+      <c r="B10" s="25"/>
+      <c r="C10" s="25"/>
+      <c r="D10" s="25"/>
+      <c r="E10" s="25"/>
+      <c r="F10" s="25"/>
+      <c r="G10" s="25"/>
+      <c r="H10" s="19" t="s">
         <v>13</v>
       </c>
-      <c r="I10" s="5" t="s">
+      <c r="I10" s="19" t="s">
         <v>14</v>
       </c>
-      <c r="J10" s="5" t="s">
+      <c r="J10" s="19" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="48"/>
-      <c r="L10" s="5" t="s">
+      <c r="K10" s="25"/>
+      <c r="L10" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="M10" s="5" t="s">
+      <c r="M10" s="19" t="s">
         <v>17</v>
       </c>
-      <c r="N10" s="5" t="s">
+      <c r="N10" s="19" t="s">
         <v>18</v>
       </c>
-      <c r="O10" s="5" t="s">
+      <c r="O10" s="19" t="s">
         <v>19</v>
       </c>
-      <c r="P10" s="5" t="s">
+      <c r="P10" s="19" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" s="54"/>
-      <c r="R10" s="55"/>
-      <c r="S10" s="48"/>
-      <c r="T10" s="48"/>
-      <c r="U10" s="48"/>
-      <c r="V10" s="51"/>
+      <c r="Q10" s="43"/>
+      <c r="R10" s="43"/>
+      <c r="S10" s="25"/>
+      <c r="T10" s="25"/>
+      <c r="U10" s="25"/>
+      <c r="V10" s="24"/>
     </row>
     <row r="11" spans="1:31" ht="15.75">
-      <c r="A11" s="6">
+      <c r="A11" s="5">
         <v>1</v>
       </c>
-      <c r="B11" s="19">
+      <c r="B11" s="18">
         <v>37074940</v>
       </c>
-      <c r="C11" s="14" t="s">
+      <c r="C11" s="13" t="s">
         <v>148</v>
       </c>
-      <c r="D11" s="19" t="s">
+      <c r="D11" s="18" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="19" t="s">
+      <c r="E11" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="F11" s="19" t="s">
+      <c r="F11" s="18" t="s">
         <v>166</v>
       </c>
-      <c r="G11" s="19">
+      <c r="G11" s="18">
         <v>10</v>
       </c>
-      <c r="H11" s="19">
+      <c r="H11" s="18">
         <v>8</v>
       </c>
-      <c r="I11" s="19" t="s">
+      <c r="I11" s="18" t="s">
         <v>176</v>
       </c>
-      <c r="J11" s="10">
+      <c r="J11" s="9">
         <v>2015</v>
       </c>
-      <c r="K11" s="56" t="s">
+      <c r="K11" s="20" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="19" t="s">
+      <c r="L11" s="18" t="s">
         <v>81</v>
       </c>
-      <c r="M11" s="19">
+      <c r="M11" s="18">
         <v>12</v>
       </c>
-      <c r="N11" s="19">
+      <c r="N11" s="18">
         <v>12</v>
       </c>
-      <c r="O11" s="19">
+      <c r="O11" s="18">
         <v>12</v>
       </c>
-      <c r="P11" s="19">
+      <c r="P11" s="18">
         <v>36</v>
       </c>
-      <c r="Q11" s="19" t="s">
+      <c r="Q11" s="18" t="s">
         <v>175</v>
       </c>
-      <c r="R11" s="19" t="s">
+      <c r="R11" s="18" t="s">
         <v>174</v>
       </c>
-      <c r="S11" s="14">
+      <c r="S11" s="13">
         <v>25886241</v>
       </c>
-      <c r="T11" s="19">
+      <c r="T11" s="18">
         <v>4262680485</v>
       </c>
-      <c r="U11" s="19" t="s">
+      <c r="U11" s="18" t="s">
         <v>173</v>
       </c>
-      <c r="V11" s="2" t="s">
+      <c r="V11" s="6" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="12" spans="1:31" ht="15.75">
-      <c r="A12" s="6">
+      <c r="A12" s="5">
         <v>2</v>
       </c>
-      <c r="B12" s="23">
+      <c r="B12" s="6">
         <v>11515295024</v>
       </c>
-      <c r="C12" s="19"/>
-      <c r="D12" s="19" t="s">
+      <c r="C12" s="18"/>
+      <c r="D12" s="18" t="s">
         <v>167</v>
       </c>
-      <c r="E12" s="19" t="s">
+      <c r="E12" s="18" t="s">
         <v>168</v>
       </c>
-      <c r="F12" s="19" t="s">
+      <c r="F12" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="G12" s="19" t="s">
+      <c r="G12" s="18" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="19">
+      <c r="H12" s="18">
         <v>24</v>
       </c>
-      <c r="I12" s="19">
+      <c r="I12" s="18">
         <v>10</v>
       </c>
-      <c r="J12" s="19">
+      <c r="J12" s="18">
         <v>2015</v>
       </c>
-      <c r="K12" s="57" t="s">
+      <c r="K12" s="21" t="s">
         <v>27</v>
       </c>
-      <c r="L12" s="19" t="s">
+      <c r="L12" s="18" t="s">
         <v>28</v>
       </c>
-      <c r="M12" s="19"/>
-      <c r="N12" s="19">
+      <c r="M12" s="18"/>
+      <c r="N12" s="18">
         <v>8</v>
       </c>
-      <c r="O12" s="19">
+      <c r="O12" s="18">
         <v>8</v>
       </c>
-      <c r="P12" s="19">
-        <v>35</v>
-      </c>
-      <c r="Q12" s="19" t="s">
+      <c r="P12" s="18">
+        <v>35</v>
+      </c>
+      <c r="Q12" s="18" t="s">
         <v>171</v>
       </c>
-      <c r="R12" s="19" t="s">
+      <c r="R12" s="18" t="s">
         <v>170</v>
       </c>
-      <c r="S12" s="19">
+      <c r="S12" s="18">
         <v>15295024</v>
       </c>
-      <c r="T12" s="19">
+      <c r="T12" s="18">
         <v>41226198111</v>
       </c>
-      <c r="U12" s="19" t="s">
+      <c r="U12" s="18" t="s">
         <v>172</v>
       </c>
-      <c r="V12" s="19" t="s">
+      <c r="V12" s="18" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="13" spans="1:31" ht="30">
-      <c r="A13" s="6">
+      <c r="A13" s="5">
         <v>3</v>
       </c>
-      <c r="B13" s="20">
+      <c r="B13" s="44">
         <v>11614588507</v>
       </c>
-      <c r="C13" s="13"/>
-      <c r="D13" s="11" t="s">
+      <c r="C13" s="12"/>
+      <c r="D13" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="11" t="s">
+      <c r="E13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H13" s="10">
+      <c r="F13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="9">
         <v>24</v>
       </c>
-      <c r="I13" s="12">
+      <c r="I13" s="11">
         <v>10</v>
       </c>
-      <c r="J13" s="12">
+      <c r="J13" s="11">
         <v>2016</v>
       </c>
-      <c r="K13" s="58" t="s">
+      <c r="K13" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L13" s="10" t="s">
+      <c r="L13" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M13" s="10"/>
-      <c r="N13" s="10">
+      <c r="M13" s="9"/>
+      <c r="N13" s="9">
         <v>10</v>
       </c>
-      <c r="O13" s="10">
+      <c r="O13" s="9">
         <v>10</v>
       </c>
-      <c r="P13" s="10">
+      <c r="P13" s="9">
         <v>36</v>
       </c>
-      <c r="Q13" s="11" t="s">
+      <c r="Q13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="R13" s="11" t="s">
+      <c r="R13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="S13" s="13">
+      <c r="S13" s="12">
         <v>14588507</v>
       </c>
-      <c r="T13" s="13" t="s">
+      <c r="T13" s="12" t="s">
         <v>46</v>
       </c>
-      <c r="U13" s="13" t="s">
+      <c r="U13" s="12" t="s">
         <v>47</v>
       </c>
-      <c r="V13" s="14" t="s">
+      <c r="V13" s="13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="14" spans="1:31" ht="30" customHeight="1">
-      <c r="A14" s="6">
+      <c r="A14" s="5">
         <v>4</v>
       </c>
-      <c r="B14" s="22">
+      <c r="B14" s="5">
         <v>11622655351</v>
       </c>
-      <c r="C14" s="11"/>
-      <c r="D14" s="18" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="17" t="s">
         <v>106</v>
       </c>
-      <c r="E14" s="11" t="s">
+      <c r="E14" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="F14" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="10">
+      <c r="F14" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="9">
         <v>16</v>
       </c>
-      <c r="I14" s="12">
+      <c r="I14" s="11">
         <v>8</v>
       </c>
-      <c r="J14" s="12">
+      <c r="J14" s="11">
         <v>2016</v>
       </c>
-      <c r="K14" s="10" t="s">
+      <c r="K14" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L14" s="10" t="s">
+      <c r="L14" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M14" s="10"/>
-      <c r="N14" s="10">
+      <c r="M14" s="9"/>
+      <c r="N14" s="9">
         <v>10</v>
       </c>
-      <c r="O14" s="10">
+      <c r="O14" s="9">
         <v>10</v>
       </c>
-      <c r="P14" s="10">
+      <c r="P14" s="9">
         <v>36</v>
       </c>
-      <c r="Q14" s="11" t="s">
+      <c r="Q14" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="R14" s="11" t="s">
+      <c r="R14" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="S14" s="11">
+      <c r="S14" s="10">
         <v>22655351</v>
       </c>
-      <c r="T14" s="11" t="s">
+      <c r="T14" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="U14" s="16" t="s">
+      <c r="U14" s="15" t="s">
         <v>111</v>
       </c>
-      <c r="V14" s="14" t="s">
+      <c r="V14" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:31" ht="30">
-      <c r="A15" s="6">
+      <c r="A15" s="5">
         <v>5</v>
       </c>
-      <c r="B15" s="22">
+      <c r="B15" s="5">
         <v>11622655622</v>
       </c>
-      <c r="C15" s="11"/>
-      <c r="D15" s="11" t="s">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="11" t="s">
+      <c r="E15" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="F15" s="11" t="s">
+      <c r="F15" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="G15" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H15" s="10">
+      <c r="G15" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="9">
         <v>3</v>
       </c>
-      <c r="I15" s="12">
+      <c r="I15" s="11">
         <v>11</v>
       </c>
-      <c r="J15" s="12">
+      <c r="J15" s="11">
         <v>2016</v>
       </c>
-      <c r="K15" s="10" t="s">
+      <c r="K15" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L15" s="10" t="s">
+      <c r="L15" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M15" s="10"/>
-      <c r="N15" s="10">
+      <c r="M15" s="9"/>
+      <c r="N15" s="9">
         <v>10</v>
       </c>
-      <c r="O15" s="10">
+      <c r="O15" s="9">
         <v>10</v>
       </c>
-      <c r="P15" s="10">
+      <c r="P15" s="9">
         <v>36</v>
       </c>
-      <c r="Q15" s="11" t="s">
+      <c r="Q15" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R15" s="11" t="s">
+      <c r="R15" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="S15" s="11">
+      <c r="S15" s="10">
         <v>22655622</v>
       </c>
-      <c r="T15" s="11" t="s">
+      <c r="T15" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="U15" s="16" t="s">
+      <c r="U15" s="15" t="s">
         <v>129</v>
       </c>
-      <c r="V15" s="14" t="s">
+      <c r="V15" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="16" spans="1:31" ht="30">
-      <c r="A16" s="6">
+      <c r="A16" s="5">
         <v>6</v>
       </c>
-      <c r="B16" s="22">
+      <c r="B16" s="5">
         <v>11625643429</v>
       </c>
-      <c r="C16" s="11"/>
-      <c r="D16" s="11" t="s">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="E16" s="11" t="s">
+      <c r="E16" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="F16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="10">
+      <c r="F16" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="9">
         <v>27</v>
       </c>
-      <c r="I16" s="12">
+      <c r="I16" s="11">
         <v>3</v>
       </c>
-      <c r="J16" s="12">
+      <c r="J16" s="11">
         <v>2016</v>
       </c>
-      <c r="K16" s="10" t="s">
+      <c r="K16" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L16" s="10" t="s">
+      <c r="L16" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M16" s="10"/>
-      <c r="N16" s="10">
+      <c r="M16" s="9"/>
+      <c r="N16" s="9">
         <v>10</v>
       </c>
-      <c r="O16" s="10">
+      <c r="O16" s="9">
         <v>10</v>
       </c>
-      <c r="P16" s="10">
+      <c r="P16" s="9">
         <v>36</v>
       </c>
-      <c r="Q16" s="11" t="s">
+      <c r="Q16" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="R16" s="11" t="s">
+      <c r="R16" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="S16" s="11">
+      <c r="S16" s="10">
         <v>25643429</v>
       </c>
-      <c r="T16" s="11" t="s">
+      <c r="T16" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="U16" s="19" t="s">
+      <c r="U16" s="18" t="s">
         <v>147</v>
       </c>
-      <c r="V16" s="14" t="s">
+      <c r="V16" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="17" spans="1:22" ht="30" customHeight="1">
-      <c r="A17" s="6">
+      <c r="A17" s="5">
         <v>7</v>
       </c>
-      <c r="B17" s="21">
+      <c r="B17" s="45">
         <v>11717129491</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="11" t="s">
+      <c r="C17" s="14"/>
+      <c r="D17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="11" t="s">
+      <c r="E17" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="11" t="s">
+      <c r="F17" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H17" s="10">
+      <c r="G17" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="9">
         <v>10</v>
       </c>
-      <c r="I17" s="12">
+      <c r="I17" s="11">
         <v>11</v>
       </c>
-      <c r="J17" s="12">
+      <c r="J17" s="11">
         <v>2017</v>
       </c>
-      <c r="K17" s="58" t="s">
+      <c r="K17" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L17" s="10" t="s">
+      <c r="L17" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M17" s="10"/>
-      <c r="N17" s="10">
+      <c r="M17" s="9"/>
+      <c r="N17" s="9">
         <v>8</v>
       </c>
-      <c r="O17" s="10">
+      <c r="O17" s="9">
         <v>8</v>
       </c>
-      <c r="P17" s="10">
+      <c r="P17" s="9">
         <v>36</v>
       </c>
-      <c r="Q17" s="11" t="s">
+      <c r="Q17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="R17" s="11" t="s">
+      <c r="R17" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="S17" s="11">
+      <c r="S17" s="10">
         <v>17129491</v>
       </c>
-      <c r="T17" s="11" t="s">
+      <c r="T17" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="U17" s="16" t="s">
+      <c r="U17" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="V17" s="14" t="s">
+      <c r="V17" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="18" spans="1:22" ht="30">
-      <c r="A18" s="6">
+      <c r="A18" s="5">
         <v>8</v>
       </c>
-      <c r="B18" s="22">
+      <c r="B18" s="5">
         <v>11717864948</v>
       </c>
-      <c r="C18" s="11"/>
-      <c r="D18" s="11" t="s">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="11" t="s">
+      <c r="E18" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="11" t="s">
+      <c r="F18" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H18" s="10">
+      <c r="G18" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="9">
         <v>26</v>
       </c>
-      <c r="I18" s="12">
+      <c r="I18" s="11">
         <v>10</v>
       </c>
-      <c r="J18" s="12">
+      <c r="J18" s="11">
         <v>2017</v>
       </c>
-      <c r="K18" s="58" t="s">
+      <c r="K18" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="10" t="s">
+      <c r="L18" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M18" s="10"/>
-      <c r="N18" s="10">
+      <c r="M18" s="9"/>
+      <c r="N18" s="9">
         <v>10</v>
       </c>
-      <c r="O18" s="10">
+      <c r="O18" s="9">
         <v>10</v>
       </c>
-      <c r="P18" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q18" s="11" t="s">
+      <c r="P18" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="R18" s="11" t="s">
+      <c r="R18" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="S18" s="11">
+      <c r="S18" s="10">
         <v>17864948</v>
       </c>
-      <c r="T18" s="11" t="s">
+      <c r="T18" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="U18" s="16" t="s">
+      <c r="U18" s="15" t="s">
         <v>61</v>
       </c>
-      <c r="V18" s="14" t="s">
+      <c r="V18" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:22" ht="30">
-      <c r="A19" s="6">
+      <c r="A19" s="5">
         <v>9</v>
       </c>
-      <c r="B19" s="22">
+      <c r="B19" s="5">
         <v>11717894774</v>
       </c>
-      <c r="C19" s="11"/>
-      <c r="D19" s="11" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E19" s="11" t="s">
+      <c r="E19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G19" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H19" s="10">
+      <c r="F19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H19" s="9">
         <v>12</v>
       </c>
-      <c r="I19" s="12">
+      <c r="I19" s="11">
         <v>12</v>
       </c>
-      <c r="J19" s="12">
+      <c r="J19" s="11">
         <v>2017</v>
       </c>
-      <c r="K19" s="58" t="s">
+      <c r="K19" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L19" s="10" t="s">
+      <c r="L19" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M19" s="10"/>
-      <c r="N19" s="10">
+      <c r="M19" s="9"/>
+      <c r="N19" s="9">
         <v>8</v>
       </c>
-      <c r="O19" s="10">
+      <c r="O19" s="9">
         <v>8</v>
       </c>
-      <c r="P19" s="10">
+      <c r="P19" s="9">
         <v>33</v>
       </c>
-      <c r="Q19" s="11" t="s">
+      <c r="Q19" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="R19" s="11" t="s">
+      <c r="R19" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S19" s="11">
+      <c r="S19" s="10">
         <v>17894774</v>
       </c>
-      <c r="T19" s="11" t="s">
+      <c r="T19" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="U19" s="16" t="s">
+      <c r="U19" s="15" t="s">
         <v>67</v>
       </c>
-      <c r="V19" s="14" t="s">
+      <c r="V19" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="20" spans="1:22" ht="30">
-      <c r="A20" s="6">
+      <c r="A20" s="5">
         <v>10</v>
       </c>
-      <c r="B20" s="22">
+      <c r="B20" s="5">
         <v>11718797834</v>
       </c>
-      <c r="C20" s="11"/>
-      <c r="D20" s="11" t="s">
+      <c r="C20" s="10"/>
+      <c r="D20" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="11" t="s">
+      <c r="E20" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G20" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H20" s="10">
+      <c r="F20" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="9">
         <v>12</v>
       </c>
-      <c r="I20" s="12">
+      <c r="I20" s="11">
         <v>10</v>
       </c>
-      <c r="J20" s="12">
+      <c r="J20" s="11">
         <v>2017</v>
       </c>
-      <c r="K20" s="10" t="s">
+      <c r="K20" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L20" s="10" t="s">
+      <c r="L20" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M20" s="10"/>
-      <c r="N20" s="10">
+      <c r="M20" s="9"/>
+      <c r="N20" s="9">
         <v>8</v>
       </c>
-      <c r="O20" s="10">
+      <c r="O20" s="9">
         <v>8</v>
       </c>
-      <c r="P20" s="10">
+      <c r="P20" s="9">
         <v>34</v>
       </c>
-      <c r="Q20" s="11" t="s">
+      <c r="Q20" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="R20" s="11" t="s">
+      <c r="R20" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="S20" s="11">
+      <c r="S20" s="10">
         <v>17864948</v>
       </c>
-      <c r="T20" s="11" t="s">
+      <c r="T20" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="U20" s="16" t="s">
+      <c r="U20" s="15" t="s">
         <v>53</v>
       </c>
-      <c r="V20" s="14" t="s">
+      <c r="V20" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="21" spans="1:22" ht="30">
-      <c r="A21" s="6">
+      <c r="A21" s="5">
         <v>11</v>
       </c>
-      <c r="B21" s="22">
+      <c r="B21" s="5">
         <v>11719071798</v>
       </c>
-      <c r="C21" s="11"/>
-      <c r="D21" s="11" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="11" t="s">
+      <c r="E21" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F21" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G21" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H21" s="10">
+      <c r="F21" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H21" s="9">
         <v>18</v>
       </c>
-      <c r="I21" s="12">
+      <c r="I21" s="11">
         <v>5</v>
       </c>
-      <c r="J21" s="12">
+      <c r="J21" s="11">
         <v>2017</v>
       </c>
-      <c r="K21" s="10" t="s">
+      <c r="K21" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L21" s="10" t="s">
+      <c r="L21" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M21" s="10"/>
-      <c r="N21" s="10">
+      <c r="M21" s="9"/>
+      <c r="N21" s="9">
         <v>8</v>
       </c>
-      <c r="O21" s="10">
+      <c r="O21" s="9">
         <v>8</v>
       </c>
-      <c r="P21" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q21" s="11" t="s">
+      <c r="P21" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q21" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="R21" s="11" t="s">
+      <c r="R21" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="S21" s="11">
+      <c r="S21" s="10">
         <v>19071798</v>
       </c>
-      <c r="T21" s="11" t="s">
+      <c r="T21" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="U21" s="16" t="s">
+      <c r="U21" s="15" t="s">
         <v>78</v>
       </c>
-      <c r="V21" s="14" t="s">
+      <c r="V21" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="22" spans="1:22" ht="30">
-      <c r="A22" s="6">
+      <c r="A22" s="5">
         <v>12</v>
       </c>
-      <c r="B22" s="22">
+      <c r="B22" s="5">
         <v>11720010470</v>
       </c>
-      <c r="C22" s="11"/>
-      <c r="D22" s="11" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E22" s="11" t="s">
+      <c r="E22" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F22" s="11" t="s">
+      <c r="F22" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="11" t="s">
+      <c r="G22" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="10">
+      <c r="H22" s="9">
         <v>7</v>
       </c>
-      <c r="I22" s="12">
+      <c r="I22" s="11">
         <v>8</v>
       </c>
-      <c r="J22" s="12">
+      <c r="J22" s="11">
         <v>2017</v>
       </c>
-      <c r="K22" s="10" t="s">
+      <c r="K22" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L22" s="10" t="s">
+      <c r="L22" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M22" s="10"/>
-      <c r="N22" s="10">
+      <c r="M22" s="9"/>
+      <c r="N22" s="9">
         <v>10</v>
       </c>
-      <c r="O22" s="10">
+      <c r="O22" s="9">
         <v>10</v>
       </c>
-      <c r="P22" s="10">
+      <c r="P22" s="9">
         <v>36</v>
       </c>
-      <c r="Q22" s="11" t="s">
+      <c r="Q22" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="R22" s="11" t="s">
+      <c r="R22" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="S22" s="11">
+      <c r="S22" s="10">
         <v>20010470</v>
       </c>
-      <c r="T22" s="11" t="s">
+      <c r="T22" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="U22" s="16" t="s">
+      <c r="U22" s="15" t="s">
         <v>105</v>
       </c>
-      <c r="V22" s="14" t="s">
+      <c r="V22" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="23" spans="1:22" ht="30">
-      <c r="A23" s="6">
+      <c r="A23" s="5">
         <v>13</v>
       </c>
-      <c r="B23" s="22">
+      <c r="B23" s="5">
         <v>11720118025</v>
       </c>
-      <c r="C23" s="11"/>
-      <c r="D23" s="11" t="s">
+      <c r="C23" s="10"/>
+      <c r="D23" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="11" t="s">
+      <c r="E23" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="11" t="s">
+      <c r="F23" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G23" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" s="10">
+      <c r="G23" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" s="9">
         <v>28</v>
       </c>
-      <c r="I23" s="12">
+      <c r="I23" s="11">
         <v>2</v>
       </c>
-      <c r="J23" s="12">
+      <c r="J23" s="11">
         <v>2017</v>
       </c>
-      <c r="K23" s="10" t="s">
+      <c r="K23" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L23" s="10" t="s">
+      <c r="L23" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M23" s="10"/>
-      <c r="N23" s="10">
+      <c r="M23" s="9"/>
+      <c r="N23" s="9">
         <v>10</v>
       </c>
-      <c r="O23" s="10">
+      <c r="O23" s="9">
         <v>10</v>
       </c>
-      <c r="P23" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q23" s="11" t="s">
+      <c r="P23" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q23" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="R23" s="11" t="s">
+      <c r="R23" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="S23" s="11">
+      <c r="S23" s="10">
         <v>20118025</v>
       </c>
-      <c r="T23" s="11" t="s">
+      <c r="T23" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="U23" s="16" t="s">
+      <c r="U23" s="15" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="14" t="s">
+      <c r="V23" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="24" spans="1:22" ht="15.75">
-      <c r="A24" s="6">
+      <c r="A24" s="5">
         <v>14</v>
       </c>
-      <c r="B24" s="22">
+      <c r="B24" s="5">
         <v>11720832435</v>
       </c>
-      <c r="C24" s="11"/>
-      <c r="D24" s="11" t="s">
+      <c r="C24" s="10"/>
+      <c r="D24" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E24" s="17" t="s">
+      <c r="E24" s="16" t="s">
         <v>80</v>
       </c>
-      <c r="F24" s="11" t="s">
+      <c r="F24" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H24" s="10">
+      <c r="G24" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="9">
         <v>10</v>
       </c>
-      <c r="I24" s="12">
+      <c r="I24" s="11">
         <v>11</v>
       </c>
-      <c r="J24" s="12">
+      <c r="J24" s="11">
         <v>2017</v>
       </c>
-      <c r="K24" s="58" t="s">
+      <c r="K24" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="10" t="s">
+      <c r="L24" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M24" s="10"/>
-      <c r="N24" s="10">
+      <c r="M24" s="9"/>
+      <c r="N24" s="9">
         <v>8</v>
       </c>
-      <c r="O24" s="10">
+      <c r="O24" s="9">
         <v>8</v>
       </c>
-      <c r="P24" s="10">
+      <c r="P24" s="9">
         <v>34</v>
       </c>
-      <c r="Q24" s="11" t="s">
+      <c r="Q24" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="R24" s="11" t="s">
+      <c r="R24" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="S24" s="11">
+      <c r="S24" s="10">
         <v>20832435</v>
       </c>
-      <c r="T24" s="11" t="s">
+      <c r="T24" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="U24" s="16" t="s">
+      <c r="U24" s="15" t="s">
         <v>85</v>
       </c>
-      <c r="V24" s="14" t="s">
+      <c r="V24" s="13" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="25" spans="1:22" ht="45">
-      <c r="A25" s="6">
+    <row r="25" spans="1:22" ht="30" customHeight="1">
+      <c r="A25" s="5">
         <v>16</v>
       </c>
-      <c r="B25" s="22">
+      <c r="B25" s="5">
         <v>11722655443</v>
       </c>
-      <c r="C25" s="11"/>
-      <c r="D25" s="11" t="s">
+      <c r="C25" s="10"/>
+      <c r="D25" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="E25" s="11" t="s">
+      <c r="E25" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="F25" s="11" t="s">
+      <c r="F25" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G25" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H25" s="10">
+      <c r="G25" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" s="9">
         <v>18</v>
       </c>
-      <c r="I25" s="12">
+      <c r="I25" s="11">
         <v>11</v>
       </c>
-      <c r="J25" s="12">
+      <c r="J25" s="11">
         <v>2017</v>
       </c>
-      <c r="K25" s="58" t="s">
+      <c r="K25" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L25" s="10" t="s">
+      <c r="L25" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M25" s="10"/>
-      <c r="N25" s="10">
+      <c r="M25" s="9"/>
+      <c r="N25" s="9">
         <v>10</v>
       </c>
-      <c r="O25" s="10">
+      <c r="O25" s="9">
         <v>10</v>
       </c>
-      <c r="P25" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q25" s="11" t="s">
+      <c r="P25" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q25" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="R25" s="11" t="s">
+      <c r="R25" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="S25" s="11">
+      <c r="S25" s="10">
         <v>9475732</v>
       </c>
-      <c r="T25" s="11" t="s">
+      <c r="T25" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="U25" s="16" t="s">
+      <c r="U25" s="15" t="s">
         <v>115</v>
       </c>
-      <c r="V25" s="14" t="s">
+      <c r="V25" s="13" t="s">
         <v>116</v>
       </c>
     </row>
     <row r="26" spans="1:22" ht="30">
-      <c r="A26" s="6">
+      <c r="A26" s="5">
         <v>17</v>
       </c>
-      <c r="B26" s="22">
+      <c r="B26" s="5">
         <v>11722655654</v>
       </c>
-      <c r="C26" s="11"/>
-      <c r="D26" s="11" t="s">
+      <c r="C26" s="10"/>
+      <c r="D26" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="11" t="s">
+      <c r="E26" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G26" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="10">
+      <c r="F26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" s="9">
         <v>17</v>
       </c>
-      <c r="I26" s="12">
+      <c r="I26" s="11">
         <v>8</v>
       </c>
-      <c r="J26" s="12">
+      <c r="J26" s="11">
         <v>2017</v>
       </c>
-      <c r="K26" s="58" t="s">
+      <c r="K26" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L26" s="10" t="s">
+      <c r="L26" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M26" s="10"/>
-      <c r="N26" s="10">
+      <c r="M26" s="9"/>
+      <c r="N26" s="9">
         <v>10</v>
       </c>
-      <c r="O26" s="10">
+      <c r="O26" s="9">
         <v>10</v>
       </c>
-      <c r="P26" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q26" s="11" t="s">
+      <c r="P26" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q26" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="R26" s="11" t="s">
+      <c r="R26" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="S26" s="11">
+      <c r="S26" s="10">
         <v>22655654</v>
       </c>
-      <c r="T26" s="11" t="s">
+      <c r="T26" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="U26" s="16" t="s">
+      <c r="U26" s="15" t="s">
         <v>122</v>
       </c>
-      <c r="V26" s="14" t="s">
+      <c r="V26" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="27" spans="1:22" ht="30">
-      <c r="A27" s="6">
+      <c r="A27" s="5">
         <v>18</v>
       </c>
-      <c r="B27" s="22">
+      <c r="B27" s="5">
         <v>11725150838</v>
       </c>
-      <c r="C27" s="11"/>
-      <c r="D27" s="11" t="s">
+      <c r="C27" s="10"/>
+      <c r="D27" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="E27" s="11" t="s">
+      <c r="E27" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="F27" s="11" t="s">
+      <c r="F27" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G27" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H27" s="10">
+      <c r="G27" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" s="9">
         <v>26</v>
       </c>
-      <c r="I27" s="12">
+      <c r="I27" s="11">
         <v>12</v>
       </c>
-      <c r="J27" s="12">
+      <c r="J27" s="11">
         <v>2017</v>
       </c>
-      <c r="K27" s="10" t="s">
+      <c r="K27" s="9" t="s">
         <v>70</v>
       </c>
-      <c r="L27" s="10" t="s">
+      <c r="L27" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M27" s="10"/>
-      <c r="N27" s="10">
+      <c r="M27" s="9"/>
+      <c r="N27" s="9">
         <v>10</v>
       </c>
-      <c r="O27" s="10">
+      <c r="O27" s="9">
         <v>10</v>
       </c>
-      <c r="P27" s="10">
-        <v>35</v>
-      </c>
-      <c r="Q27" s="11" t="s">
+      <c r="P27" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q27" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="R27" s="11" t="s">
+      <c r="R27" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="S27" s="11">
+      <c r="S27" s="10">
         <v>25150838</v>
       </c>
-      <c r="T27" s="11" t="s">
+      <c r="T27" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="U27" s="16" t="s">
+      <c r="U27" s="15" t="s">
         <v>135</v>
       </c>
-      <c r="V27" s="14" t="s">
+      <c r="V27" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="28" spans="1:22" ht="30">
-      <c r="A28" s="6">
+      <c r="A28" s="5">
         <v>19</v>
       </c>
-      <c r="B28" s="22">
+      <c r="B28" s="5">
         <v>11725643421</v>
       </c>
-      <c r="C28" s="11"/>
-      <c r="D28" s="11" t="s">
+      <c r="C28" s="10"/>
+      <c r="D28" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="E28" s="11" t="s">
+      <c r="E28" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="F28" s="11" t="s">
+      <c r="F28" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H28" s="10">
+      <c r="G28" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" s="9">
         <v>4</v>
       </c>
-      <c r="I28" s="12">
+      <c r="I28" s="11">
         <v>12</v>
       </c>
-      <c r="J28" s="12">
+      <c r="J28" s="11">
         <v>2017</v>
       </c>
-      <c r="K28" s="58" t="s">
+      <c r="K28" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L28" s="10" t="s">
+      <c r="L28" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M28" s="10"/>
-      <c r="N28" s="10">
+      <c r="M28" s="9"/>
+      <c r="N28" s="9">
         <v>8</v>
       </c>
-      <c r="O28" s="10">
+      <c r="O28" s="9">
         <v>8</v>
       </c>
-      <c r="P28" s="10">
+      <c r="P28" s="9">
         <v>34</v>
       </c>
-      <c r="Q28" s="11" t="s">
+      <c r="Q28" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="R28" s="11" t="s">
+      <c r="R28" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="S28" s="11">
+      <c r="S28" s="10">
         <v>25643421</v>
       </c>
-      <c r="T28" s="11" t="s">
+      <c r="T28" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="U28" s="16" t="s">
+      <c r="U28" s="15" t="s">
         <v>141</v>
       </c>
-      <c r="V28" s="14" t="s">
+      <c r="V28" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="29" spans="1:22" ht="30" customHeight="1">
-      <c r="A29" s="6">
+      <c r="A29" s="5">
         <v>20</v>
       </c>
-      <c r="B29" s="21">
+      <c r="B29" s="45">
         <v>11814699917</v>
       </c>
-      <c r="C29" s="15"/>
-      <c r="D29" s="11" t="s">
+      <c r="C29" s="14"/>
+      <c r="D29" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E29" s="11" t="s">
+      <c r="E29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F29" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G29" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="H29" s="10">
+      <c r="F29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H29" s="9">
         <v>5</v>
       </c>
-      <c r="I29" s="12">
+      <c r="I29" s="11">
         <v>1</v>
       </c>
-      <c r="J29" s="12">
+      <c r="J29" s="11">
         <v>2017</v>
       </c>
-      <c r="K29" s="58" t="s">
+      <c r="K29" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L29" s="10" t="s">
+      <c r="L29" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M29" s="10"/>
-      <c r="N29" s="10">
+      <c r="M29" s="9"/>
+      <c r="N29" s="9">
         <v>8</v>
       </c>
-      <c r="O29" s="10">
+      <c r="O29" s="9">
         <v>8</v>
       </c>
-      <c r="P29" s="10">
+      <c r="P29" s="9">
         <v>34</v>
       </c>
-      <c r="Q29" s="11" t="s">
+      <c r="Q29" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="R29" s="11" t="s">
+      <c r="R29" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="S29" s="15">
+      <c r="S29" s="14">
         <v>14699917</v>
       </c>
-      <c r="T29" s="15" t="s">
+      <c r="T29" s="14" t="s">
         <v>32</v>
       </c>
-      <c r="U29" s="15" t="s">
+      <c r="U29" s="14" t="s">
         <v>33</v>
       </c>
-      <c r="V29" s="14" t="s">
+      <c r="V29" s="13" t="s">
         <v>31</v>
       </c>
     </row>
     <row r="30" spans="1:22" ht="30">
-      <c r="A30" s="9">
+      <c r="A30" s="8">
         <v>21</v>
       </c>
-      <c r="B30" s="22">
+      <c r="B30" s="5">
         <v>11820435077</v>
       </c>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25" t="s">
+      <c r="C30" s="10"/>
+      <c r="D30" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="25" t="s">
+      <c r="E30" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="F30" s="25" t="s">
+      <c r="F30" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G30" s="25" t="s">
-        <v>35</v>
-      </c>
-      <c r="H30" s="26">
+      <c r="G30" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H30" s="9">
         <v>26</v>
       </c>
-      <c r="I30" s="27">
+      <c r="I30" s="11">
         <v>1</v>
       </c>
-      <c r="J30" s="27">
+      <c r="J30" s="11">
         <v>2018</v>
       </c>
-      <c r="K30" s="59" t="s">
+      <c r="K30" s="22" t="s">
         <v>27</v>
       </c>
-      <c r="L30" s="26" t="s">
+      <c r="L30" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="M30" s="26"/>
-      <c r="N30" s="26">
+      <c r="M30" s="9"/>
+      <c r="N30" s="9">
         <v>8</v>
       </c>
-      <c r="O30" s="26">
+      <c r="O30" s="9">
         <v>8</v>
       </c>
-      <c r="P30" s="26">
+      <c r="P30" s="9">
         <v>34</v>
       </c>
-      <c r="Q30" s="25" t="s">
+      <c r="Q30" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="R30" s="28" t="s">
+      <c r="R30" s="16" t="s">
         <v>89</v>
       </c>
-      <c r="S30" s="25">
+      <c r="S30" s="10">
         <v>20435077</v>
       </c>
-      <c r="T30" s="25" t="s">
+      <c r="T30" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="U30" s="29" t="s">
+      <c r="U30" s="15" t="s">
         <v>91</v>
       </c>
-      <c r="V30" s="30" t="s">
+      <c r="V30" s="13" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="31" spans="1:22" ht="15.75" customHeight="1">
-      <c r="A31" s="2">
+      <c r="A31" s="46">
         <v>22</v>
       </c>
-      <c r="B31" s="24"/>
-      <c r="C31" s="7"/>
-      <c r="D31" s="7"/>
-      <c r="E31" s="7"/>
-      <c r="F31" s="7"/>
-      <c r="G31" s="7"/>
-      <c r="H31" s="7"/>
-      <c r="I31" s="7"/>
-      <c r="J31" s="7"/>
-      <c r="K31" s="7"/>
-      <c r="L31" s="7"/>
-      <c r="M31" s="7"/>
-      <c r="N31" s="7"/>
-      <c r="O31" s="7"/>
-      <c r="P31" s="7"/>
-      <c r="Q31" s="7"/>
-      <c r="R31" s="7"/>
-      <c r="S31" s="7"/>
-      <c r="T31" s="7"/>
-      <c r="U31" s="7"/>
-      <c r="V31" s="7"/>
-    </row>
-    <row r="38" spans="1:21" ht="30">
-      <c r="A38" s="20">
+      <c r="B31" s="44">
         <v>11313966325</v>
       </c>
-      <c r="B38" s="11"/>
-      <c r="C38" s="11" t="s">
+      <c r="C31" s="10"/>
+      <c r="D31" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="D38" s="11" t="s">
+      <c r="E31" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="E38" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="F38" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="G38" s="10">
+      <c r="F31" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H31" s="9">
         <v>15</v>
       </c>
-      <c r="H38" s="12">
+      <c r="I31" s="11">
         <v>8</v>
       </c>
-      <c r="I38" s="12">
+      <c r="J31" s="11">
         <v>2017</v>
       </c>
-      <c r="J38" s="60" t="s">
+      <c r="K31" s="23" t="s">
         <v>27</v>
       </c>
-      <c r="K38" s="10" t="s">
+      <c r="L31" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="L38" s="10"/>
-      <c r="M38" s="10">
+      <c r="M31" s="9"/>
+      <c r="N31" s="9">
         <v>8</v>
       </c>
-      <c r="N38" s="10">
+      <c r="O31" s="9">
         <v>8</v>
       </c>
-      <c r="O38" s="10">
-        <v>35</v>
-      </c>
-      <c r="P38" s="11" t="s">
+      <c r="P31" s="9">
+        <v>35</v>
+      </c>
+      <c r="Q31" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="Q38" s="11" t="s">
+      <c r="R31" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="R38" s="11">
+      <c r="S31" s="10">
         <v>13966325</v>
       </c>
-      <c r="S38" s="13" t="s">
+      <c r="T31" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="T38" s="13" t="s">
+      <c r="U31" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="U38" s="14" t="s">
+      <c r="V31" s="13" t="s">
         <v>54</v>
       </c>
     </row>
@@ -2966,32 +2870,6 @@
     <sortCondition ref="B11"/>
   </sortState>
   <mergeCells count="40">
-    <mergeCell ref="V9:V10"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="Q9:R10"/>
-    <mergeCell ref="D9:E10"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="A8:P8"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="Q8:V8"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="K7:L7"/>
     <mergeCell ref="W5:X5"/>
     <mergeCell ref="Z5:AB5"/>
     <mergeCell ref="AD5:AE5"/>
@@ -3006,6 +2884,32 @@
     <mergeCell ref="AD6:AE6"/>
     <mergeCell ref="S6:V6"/>
     <mergeCell ref="A5:V5"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="AB7:AD7"/>
+    <mergeCell ref="A8:P8"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="Q8:V8"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="D9:E10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="Q9:R10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>

<commit_message>
coreccion del primer estudiante del trecer grado, poseia cedula de identidad, pero se extajeron mal los datos al cvs
</commit_message>
<xml_diff>
--- a/Matricula_3er_grado.xlsx
+++ b/Matricula_3er_grado.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Usuario\Documents\Project\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A660B5DE-3771-465E-9318-A0C8866E27DD}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A351825C-909F-437E-930D-2DF32374A6F2}" xr6:coauthVersionLast="43" xr6:coauthVersionMax="43" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="21840" windowHeight="13140" tabRatio="278" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="274" uniqueCount="177">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="273" uniqueCount="177">
   <si>
     <t>Código plan de estudio:</t>
   </si>
@@ -564,7 +564,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="8">
+  <fonts count="9">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -614,6 +614,13 @@
       <family val="2"/>
     </font>
     <font>
+      <sz val="12"/>
+      <color theme="1"/>
+      <name val="Arial Narrow"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <u/>
       <sz val="12"/>
       <color theme="1"/>
       <name val="Arial Narrow"/>
@@ -763,7 +770,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="39">
+  <cellXfs count="41">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="justify" vertical="top" wrapText="1"/>
@@ -779,66 +786,6 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="justify" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
@@ -870,6 +817,70 @@
     </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="justify" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1225,165 +1236,165 @@
   </cols>
   <sheetData>
     <row r="5" spans="1:31" ht="30.95" customHeight="1">
-      <c r="A5" s="13" t="s">
+      <c r="A5" s="37" t="s">
         <v>26</v>
       </c>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14"/>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14"/>
-      <c r="G5" s="14"/>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14"/>
-      <c r="U5" s="14"/>
-      <c r="V5" s="14"/>
-      <c r="W5" s="7"/>
-      <c r="X5" s="7"/>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+      <c r="J5" s="38"/>
+      <c r="K5" s="38"/>
+      <c r="L5" s="38"/>
+      <c r="M5" s="38"/>
+      <c r="N5" s="38"/>
+      <c r="O5" s="38"/>
+      <c r="P5" s="38"/>
+      <c r="Q5" s="38"/>
+      <c r="R5" s="38"/>
+      <c r="S5" s="38"/>
+      <c r="T5" s="38"/>
+      <c r="U5" s="38"/>
+      <c r="V5" s="38"/>
+      <c r="W5" s="23"/>
+      <c r="X5" s="23"/>
       <c r="Y5" s="1"/>
-      <c r="Z5" s="7"/>
-      <c r="AA5" s="7"/>
-      <c r="AB5" s="7"/>
+      <c r="Z5" s="23"/>
+      <c r="AA5" s="23"/>
+      <c r="AB5" s="23"/>
       <c r="AC5" s="1"/>
-      <c r="AD5" s="7"/>
-      <c r="AE5" s="7"/>
+      <c r="AD5" s="23"/>
+      <c r="AE5" s="23"/>
     </row>
     <row r="6" spans="1:31" ht="27.95" customHeight="1">
-      <c r="A6" s="8" t="s">
+      <c r="A6" s="32" t="s">
         <v>150</v>
       </c>
-      <c r="B6" s="8"/>
-      <c r="C6" s="8" t="s">
+      <c r="B6" s="32"/>
+      <c r="C6" s="32" t="s">
         <v>151</v>
       </c>
-      <c r="D6" s="8"/>
-      <c r="E6" s="8" t="s">
+      <c r="D6" s="32"/>
+      <c r="E6" s="32" t="s">
         <v>152</v>
       </c>
-      <c r="F6" s="8"/>
-      <c r="G6" s="8"/>
-      <c r="H6" s="8"/>
-      <c r="I6" s="8" t="s">
+      <c r="F6" s="32"/>
+      <c r="G6" s="32"/>
+      <c r="H6" s="32"/>
+      <c r="I6" s="32" t="s">
         <v>153</v>
       </c>
-      <c r="J6" s="8"/>
-      <c r="K6" s="8"/>
-      <c r="L6" s="8"/>
-      <c r="M6" s="8" t="s">
+      <c r="J6" s="32"/>
+      <c r="K6" s="32"/>
+      <c r="L6" s="32"/>
+      <c r="M6" s="32" t="s">
         <v>154</v>
       </c>
-      <c r="N6" s="8"/>
-      <c r="O6" s="8"/>
-      <c r="P6" s="8"/>
-      <c r="Q6" s="8" t="s">
+      <c r="N6" s="32"/>
+      <c r="O6" s="32"/>
+      <c r="P6" s="32"/>
+      <c r="Q6" s="32" t="s">
         <v>155</v>
       </c>
-      <c r="R6" s="8"/>
-      <c r="S6" s="10" t="s">
+      <c r="R6" s="32"/>
+      <c r="S6" s="34" t="s">
         <v>156</v>
       </c>
-      <c r="T6" s="11"/>
-      <c r="U6" s="11"/>
-      <c r="V6" s="12"/>
-      <c r="W6" s="7"/>
-      <c r="X6" s="7"/>
-      <c r="Z6" s="9"/>
-      <c r="AA6" s="9"/>
-      <c r="AB6" s="9"/>
+      <c r="T6" s="35"/>
+      <c r="U6" s="35"/>
+      <c r="V6" s="36"/>
+      <c r="W6" s="23"/>
+      <c r="X6" s="23"/>
+      <c r="Z6" s="33"/>
+      <c r="AA6" s="33"/>
+      <c r="AB6" s="33"/>
       <c r="AC6" s="1"/>
-      <c r="AD6" s="9"/>
-      <c r="AE6" s="9"/>
+      <c r="AD6" s="33"/>
+      <c r="AE6" s="33"/>
     </row>
     <row r="7" spans="1:31" ht="36" customHeight="1">
-      <c r="A7" s="21" t="s">
+      <c r="A7" s="29" t="s">
         <v>164</v>
       </c>
-      <c r="B7" s="22"/>
-      <c r="C7" s="23"/>
-      <c r="D7" s="15" t="s">
+      <c r="B7" s="30"/>
+      <c r="C7" s="31"/>
+      <c r="D7" s="22" t="s">
         <v>163</v>
       </c>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15" t="s">
+      <c r="E7" s="22"/>
+      <c r="F7" s="22" t="s">
         <v>0</v>
       </c>
-      <c r="G7" s="15"/>
-      <c r="H7" s="15" t="s">
+      <c r="G7" s="22"/>
+      <c r="H7" s="22" t="s">
         <v>162</v>
       </c>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="21" t="s">
+      <c r="I7" s="22"/>
+      <c r="J7" s="22"/>
+      <c r="K7" s="29" t="s">
         <v>161</v>
       </c>
-      <c r="L7" s="23"/>
-      <c r="M7" s="15" t="s">
+      <c r="L7" s="31"/>
+      <c r="M7" s="22" t="s">
         <v>160</v>
       </c>
-      <c r="N7" s="15"/>
-      <c r="O7" s="15" t="s">
+      <c r="N7" s="22"/>
+      <c r="O7" s="22" t="s">
         <v>159</v>
       </c>
-      <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
+      <c r="P7" s="22"/>
+      <c r="Q7" s="22"/>
+      <c r="R7" s="22"/>
       <c r="S7" s="5" t="s">
         <v>158</v>
       </c>
       <c r="T7" s="5" t="s">
         <v>157</v>
       </c>
-      <c r="U7" s="17" t="s">
+      <c r="U7" s="25" t="s">
         <v>165</v>
       </c>
-      <c r="V7" s="18"/>
+      <c r="V7" s="26"/>
       <c r="W7" s="3"/>
       <c r="AA7" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="AB7" s="7"/>
-      <c r="AC7" s="7"/>
-      <c r="AD7" s="7"/>
+      <c r="AB7" s="23"/>
+      <c r="AC7" s="23"/>
+      <c r="AD7" s="23"/>
       <c r="AE7" s="4"/>
     </row>
     <row r="8" spans="1:31" ht="17.100000000000001" customHeight="1">
-      <c r="A8" s="16" t="s">
+      <c r="A8" s="24" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="16"/>
-      <c r="C8" s="16"/>
-      <c r="D8" s="16"/>
-      <c r="E8" s="16"/>
-      <c r="F8" s="16"/>
-      <c r="G8" s="16"/>
-      <c r="H8" s="16"/>
-      <c r="I8" s="16"/>
-      <c r="J8" s="16"/>
-      <c r="K8" s="16"/>
-      <c r="L8" s="16"/>
-      <c r="M8" s="16"/>
-      <c r="N8" s="16"/>
-      <c r="O8" s="16"/>
-      <c r="P8" s="16"/>
-      <c r="Q8" s="19" t="s">
+      <c r="B8" s="24"/>
+      <c r="C8" s="24"/>
+      <c r="D8" s="24"/>
+      <c r="E8" s="24"/>
+      <c r="F8" s="24"/>
+      <c r="G8" s="24"/>
+      <c r="H8" s="24"/>
+      <c r="I8" s="24"/>
+      <c r="J8" s="24"/>
+      <c r="K8" s="24"/>
+      <c r="L8" s="24"/>
+      <c r="M8" s="24"/>
+      <c r="N8" s="24"/>
+      <c r="O8" s="24"/>
+      <c r="P8" s="24"/>
+      <c r="Q8" s="27" t="s">
         <v>3</v>
       </c>
-      <c r="R8" s="20"/>
-      <c r="S8" s="20"/>
-      <c r="T8" s="20"/>
-      <c r="U8" s="20"/>
-      <c r="V8" s="20"/>
+      <c r="R8" s="28"/>
+      <c r="S8" s="28"/>
+      <c r="T8" s="28"/>
+      <c r="U8" s="28"/>
+      <c r="V8" s="28"/>
       <c r="W8" s="4"/>
       <c r="X8" s="1"/>
       <c r="Y8" s="1"/>
@@ -1395,67 +1406,67 @@
       <c r="AE8" s="4"/>
     </row>
     <row r="9" spans="1:31" ht="15">
-      <c r="A9" s="24" t="s">
+      <c r="A9" s="20" t="s">
         <v>4</v>
       </c>
-      <c r="B9" s="24" t="s">
+      <c r="B9" s="20" t="s">
         <v>5</v>
       </c>
-      <c r="C9" s="24" t="s">
+      <c r="C9" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="D9" s="24" t="s">
+      <c r="D9" s="20" t="s">
         <v>7</v>
       </c>
-      <c r="E9" s="24"/>
-      <c r="F9" s="24" t="s">
+      <c r="E9" s="20"/>
+      <c r="F9" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="G9" s="24" t="s">
+      <c r="G9" s="20" t="s">
         <v>8</v>
       </c>
-      <c r="H9" s="24" t="s">
+      <c r="H9" s="20" t="s">
         <v>9</v>
       </c>
-      <c r="I9" s="24"/>
-      <c r="J9" s="24"/>
-      <c r="K9" s="24" t="s">
+      <c r="I9" s="20"/>
+      <c r="J9" s="20"/>
+      <c r="K9" s="20" t="s">
         <v>10</v>
       </c>
-      <c r="L9" s="24" t="s">
+      <c r="L9" s="20" t="s">
         <v>11</v>
       </c>
-      <c r="M9" s="24"/>
-      <c r="N9" s="24" t="s">
+      <c r="M9" s="20"/>
+      <c r="N9" s="20" t="s">
         <v>22</v>
       </c>
-      <c r="O9" s="24"/>
-      <c r="P9" s="24"/>
-      <c r="Q9" s="26" t="s">
+      <c r="O9" s="20"/>
+      <c r="P9" s="20"/>
+      <c r="Q9" s="21" t="s">
         <v>12</v>
       </c>
-      <c r="R9" s="26"/>
-      <c r="S9" s="24" t="s">
+      <c r="R9" s="21"/>
+      <c r="S9" s="20" t="s">
         <v>6</v>
       </c>
-      <c r="T9" s="24" t="s">
+      <c r="T9" s="20" t="s">
         <v>23</v>
       </c>
-      <c r="U9" s="24" t="s">
+      <c r="U9" s="20" t="s">
         <v>24</v>
       </c>
-      <c r="V9" s="25" t="s">
+      <c r="V9" s="19" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="10" spans="1:31" ht="15">
-      <c r="A10" s="24"/>
-      <c r="B10" s="24"/>
-      <c r="C10" s="24"/>
-      <c r="D10" s="24"/>
-      <c r="E10" s="24"/>
-      <c r="F10" s="24"/>
-      <c r="G10" s="24"/>
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+      <c r="C10" s="20"/>
+      <c r="D10" s="20"/>
+      <c r="E10" s="20"/>
+      <c r="F10" s="20"/>
+      <c r="G10" s="20"/>
       <c r="H10" s="6" t="s">
         <v>13</v>
       </c>
@@ -1465,7 +1476,7 @@
       <c r="J10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="K10" s="24"/>
+      <c r="K10" s="20"/>
       <c r="L10" s="6" t="s">
         <v>16</v>
       </c>
@@ -1481,1536 +1492,1507 @@
       <c r="P10" s="6" t="s">
         <v>20</v>
       </c>
-      <c r="Q10" s="26"/>
-      <c r="R10" s="26"/>
-      <c r="S10" s="24"/>
-      <c r="T10" s="24"/>
-      <c r="U10" s="24"/>
-      <c r="V10" s="25"/>
+      <c r="Q10" s="21"/>
+      <c r="R10" s="21"/>
+      <c r="S10" s="20"/>
+      <c r="T10" s="20"/>
+      <c r="U10" s="20"/>
+      <c r="V10" s="19"/>
     </row>
     <row r="11" spans="1:31" ht="15.75">
-      <c r="A11" s="30">
+      <c r="A11" s="10">
         <v>1</v>
       </c>
-      <c r="B11" s="27">
+      <c r="C11" s="39">
         <v>37074940</v>
       </c>
-      <c r="C11" s="28" t="s">
+      <c r="D11" s="40" t="s">
         <v>148</v>
       </c>
-      <c r="D11" s="27" t="s">
+      <c r="E11" s="39" t="s">
         <v>149</v>
       </c>
-      <c r="E11" s="27" t="s">
+      <c r="F11" s="7" t="s">
         <v>166</v>
       </c>
-      <c r="F11" s="27" t="s">
-        <v>166</v>
-      </c>
-      <c r="G11" s="27">
+      <c r="G11" s="7">
         <v>10</v>
       </c>
-      <c r="H11" s="27">
+      <c r="H11" s="7">
         <v>8</v>
       </c>
-      <c r="I11" s="27" t="s">
+      <c r="I11" s="7" t="s">
         <v>176</v>
       </c>
-      <c r="J11" s="30">
+      <c r="J11" s="10">
         <v>2015</v>
       </c>
-      <c r="K11" s="37" t="s">
+      <c r="K11" s="17" t="s">
         <v>27</v>
       </c>
-      <c r="L11" s="27" t="s">
+      <c r="L11" s="7" t="s">
         <v>81</v>
       </c>
-      <c r="M11" s="27">
+      <c r="M11" s="7">
         <v>12</v>
       </c>
-      <c r="N11" s="27">
+      <c r="N11" s="7">
         <v>12</v>
       </c>
-      <c r="O11" s="27">
+      <c r="O11" s="7">
         <v>12</v>
       </c>
-      <c r="P11" s="27">
+      <c r="P11" s="7">
         <v>36</v>
       </c>
-      <c r="Q11" s="27" t="s">
+      <c r="Q11" s="7" t="s">
         <v>175</v>
       </c>
-      <c r="R11" s="27" t="s">
+      <c r="R11" s="7" t="s">
         <v>174</v>
       </c>
-      <c r="S11" s="28">
+      <c r="S11" s="8">
         <v>25886241</v>
       </c>
-      <c r="T11" s="27">
+      <c r="T11" s="7">
         <v>4262680485</v>
       </c>
-      <c r="U11" s="27" t="s">
+      <c r="U11" s="7" t="s">
         <v>173</v>
       </c>
-      <c r="V11" s="27" t="s">
+      <c r="V11" s="7" t="s">
         <v>54</v>
       </c>
-      <c r="W11" s="35"/>
-      <c r="X11" s="35"/>
-      <c r="Y11" s="35"/>
+      <c r="W11" s="15"/>
+      <c r="X11" s="15"/>
+      <c r="Y11" s="15"/>
     </row>
     <row r="12" spans="1:31" ht="15.75">
-      <c r="A12" s="30">
+      <c r="A12" s="10">
         <v>2</v>
       </c>
-      <c r="B12" s="27">
+      <c r="B12" s="7">
         <v>11515295024</v>
       </c>
-      <c r="C12" s="27"/>
-      <c r="D12" s="27" t="s">
+      <c r="C12" s="7"/>
+      <c r="D12" s="7" t="s">
         <v>167</v>
       </c>
-      <c r="E12" s="27" t="s">
+      <c r="E12" s="7" t="s">
         <v>168</v>
       </c>
-      <c r="F12" s="27" t="s">
+      <c r="F12" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="G12" s="27" t="s">
+      <c r="G12" s="7" t="s">
         <v>169</v>
       </c>
-      <c r="H12" s="27">
+      <c r="H12" s="7">
         <v>24</v>
       </c>
-      <c r="I12" s="27">
+      <c r="I12" s="7">
         <v>10</v>
       </c>
-      <c r="J12" s="27">
+      <c r="J12" s="7">
         <v>2015</v>
       </c>
-      <c r="K12" s="34" t="s">
+      <c r="K12" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="L12" s="27" t="s">
+      <c r="L12" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="M12" s="27"/>
-      <c r="N12" s="27">
+      <c r="M12" s="7"/>
+      <c r="N12" s="7">
         <v>8</v>
       </c>
-      <c r="O12" s="27">
+      <c r="O12" s="7">
         <v>8</v>
       </c>
-      <c r="P12" s="27">
-        <v>35</v>
-      </c>
-      <c r="Q12" s="27" t="s">
+      <c r="P12" s="7">
+        <v>35</v>
+      </c>
+      <c r="Q12" s="7" t="s">
         <v>171</v>
       </c>
-      <c r="R12" s="27" t="s">
+      <c r="R12" s="7" t="s">
         <v>170</v>
       </c>
-      <c r="S12" s="27">
+      <c r="S12" s="7">
         <v>15295024</v>
       </c>
-      <c r="T12" s="27">
+      <c r="T12" s="7">
         <v>41226198111</v>
       </c>
-      <c r="U12" s="27" t="s">
+      <c r="U12" s="7" t="s">
         <v>172</v>
       </c>
-      <c r="V12" s="27" t="s">
+      <c r="V12" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="W12" s="35"/>
-      <c r="X12" s="35"/>
-      <c r="Y12" s="35"/>
+      <c r="W12" s="15"/>
+      <c r="X12" s="15"/>
+      <c r="Y12" s="15"/>
     </row>
     <row r="13" spans="1:31" ht="15.75">
-      <c r="A13" s="30">
+      <c r="A13" s="10">
         <v>3</v>
       </c>
-      <c r="B13" s="29">
+      <c r="B13" s="9">
         <v>11614588507</v>
       </c>
-      <c r="C13" s="29"/>
-      <c r="D13" s="30" t="s">
+      <c r="C13" s="9"/>
+      <c r="D13" s="10" t="s">
         <v>42</v>
       </c>
-      <c r="E13" s="30" t="s">
+      <c r="E13" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="F13" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G13" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H13" s="30">
+      <c r="F13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G13" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H13" s="10">
         <v>24</v>
       </c>
-      <c r="I13" s="31">
+      <c r="I13" s="11">
         <v>10</v>
       </c>
-      <c r="J13" s="31">
+      <c r="J13" s="11">
         <v>2016</v>
       </c>
-      <c r="K13" s="38" t="s">
+      <c r="K13" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L13" s="30" t="s">
+      <c r="L13" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M13" s="30"/>
-      <c r="N13" s="30">
+      <c r="M13" s="10"/>
+      <c r="N13" s="10">
         <v>10</v>
       </c>
-      <c r="O13" s="30">
+      <c r="O13" s="10">
         <v>10</v>
       </c>
-      <c r="P13" s="30">
+      <c r="P13" s="10">
         <v>36</v>
       </c>
-      <c r="Q13" s="30" t="s">
+      <c r="Q13" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="R13" s="30" t="s">
+      <c r="R13" s="10" t="s">
         <v>45</v>
       </c>
-      <c r="S13" s="29">
+      <c r="S13" s="9">
         <v>14588507</v>
       </c>
-      <c r="T13" s="29" t="s">
+      <c r="T13" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="U13" s="29" t="s">
+      <c r="U13" s="9" t="s">
         <v>47</v>
       </c>
-      <c r="V13" s="28" t="s">
+      <c r="V13" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="W13" s="35"/>
-      <c r="X13" s="35"/>
-      <c r="Y13" s="35"/>
+      <c r="W13" s="15"/>
+      <c r="X13" s="15"/>
+      <c r="Y13" s="15"/>
     </row>
     <row r="14" spans="1:31" ht="30" customHeight="1">
-      <c r="A14" s="30">
+      <c r="A14" s="10">
         <v>4</v>
       </c>
-      <c r="B14" s="30">
+      <c r="B14" s="10">
         <v>11622655351</v>
       </c>
-      <c r="C14" s="30"/>
-      <c r="D14" s="31" t="s">
+      <c r="C14" s="10"/>
+      <c r="D14" s="11" t="s">
         <v>106</v>
       </c>
-      <c r="E14" s="30" t="s">
+      <c r="E14" s="10" t="s">
         <v>107</v>
       </c>
-      <c r="F14" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G14" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H14" s="30">
+      <c r="F14" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H14" s="10">
         <v>16</v>
       </c>
-      <c r="I14" s="31">
+      <c r="I14" s="11">
         <v>8</v>
       </c>
-      <c r="J14" s="31">
+      <c r="J14" s="11">
         <v>2016</v>
       </c>
-      <c r="K14" s="30" t="s">
+      <c r="K14" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L14" s="30" t="s">
+      <c r="L14" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M14" s="30"/>
-      <c r="N14" s="30">
+      <c r="M14" s="10"/>
+      <c r="N14" s="10">
         <v>10</v>
       </c>
-      <c r="O14" s="30">
+      <c r="O14" s="10">
         <v>10</v>
       </c>
-      <c r="P14" s="30">
+      <c r="P14" s="10">
         <v>36</v>
       </c>
-      <c r="Q14" s="30" t="s">
+      <c r="Q14" s="10" t="s">
         <v>108</v>
       </c>
-      <c r="R14" s="30" t="s">
+      <c r="R14" s="10" t="s">
         <v>109</v>
       </c>
-      <c r="S14" s="30">
+      <c r="S14" s="10">
         <v>22655351</v>
       </c>
-      <c r="T14" s="30" t="s">
+      <c r="T14" s="10" t="s">
         <v>110</v>
       </c>
-      <c r="U14" s="32" t="s">
+      <c r="U14" s="12" t="s">
         <v>111</v>
       </c>
-      <c r="V14" s="28" t="s">
+      <c r="V14" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W14" s="35"/>
-      <c r="X14" s="35"/>
-      <c r="Y14" s="35"/>
+      <c r="W14" s="15"/>
+      <c r="X14" s="15"/>
+      <c r="Y14" s="15"/>
     </row>
     <row r="15" spans="1:31" ht="31.5">
-      <c r="A15" s="30">
+      <c r="A15" s="10">
         <v>5</v>
       </c>
-      <c r="B15" s="30">
+      <c r="B15" s="10">
         <v>11622655622</v>
       </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="30" t="s">
+      <c r="C15" s="10"/>
+      <c r="D15" s="10" t="s">
         <v>123</v>
       </c>
-      <c r="E15" s="30" t="s">
+      <c r="E15" s="10" t="s">
         <v>124</v>
       </c>
-      <c r="F15" s="30" t="s">
+      <c r="F15" s="10" t="s">
         <v>125</v>
       </c>
-      <c r="G15" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H15" s="30">
+      <c r="G15" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H15" s="10">
         <v>3</v>
       </c>
-      <c r="I15" s="31">
+      <c r="I15" s="11">
         <v>11</v>
       </c>
-      <c r="J15" s="31">
+      <c r="J15" s="11">
         <v>2016</v>
       </c>
-      <c r="K15" s="30" t="s">
+      <c r="K15" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L15" s="30" t="s">
+      <c r="L15" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M15" s="30"/>
-      <c r="N15" s="30">
+      <c r="M15" s="10"/>
+      <c r="N15" s="10">
         <v>10</v>
       </c>
-      <c r="O15" s="30">
+      <c r="O15" s="10">
         <v>10</v>
       </c>
-      <c r="P15" s="30">
+      <c r="P15" s="10">
         <v>36</v>
       </c>
-      <c r="Q15" s="30" t="s">
+      <c r="Q15" s="10" t="s">
         <v>126</v>
       </c>
-      <c r="R15" s="30" t="s">
+      <c r="R15" s="10" t="s">
         <v>127</v>
       </c>
-      <c r="S15" s="30">
+      <c r="S15" s="10">
         <v>22655622</v>
       </c>
-      <c r="T15" s="30" t="s">
+      <c r="T15" s="10" t="s">
         <v>128</v>
       </c>
-      <c r="U15" s="32" t="s">
+      <c r="U15" s="12" t="s">
         <v>129</v>
       </c>
-      <c r="V15" s="28" t="s">
+      <c r="V15" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W15" s="35"/>
-      <c r="X15" s="35"/>
-      <c r="Y15" s="35"/>
+      <c r="W15" s="15"/>
+      <c r="X15" s="15"/>
+      <c r="Y15" s="15"/>
     </row>
     <row r="16" spans="1:31" ht="15.75">
-      <c r="A16" s="30">
+      <c r="A16" s="10">
         <v>6</v>
       </c>
-      <c r="B16" s="30">
+      <c r="B16" s="10">
         <v>11625643429</v>
       </c>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30" t="s">
+      <c r="C16" s="10"/>
+      <c r="D16" s="10" t="s">
         <v>142</v>
       </c>
-      <c r="E16" s="30" t="s">
+      <c r="E16" s="10" t="s">
         <v>143</v>
       </c>
-      <c r="F16" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G16" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H16" s="30">
+      <c r="F16" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G16" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H16" s="10">
         <v>27</v>
       </c>
-      <c r="I16" s="31">
+      <c r="I16" s="11">
         <v>3</v>
       </c>
-      <c r="J16" s="31">
+      <c r="J16" s="11">
         <v>2016</v>
       </c>
-      <c r="K16" s="30" t="s">
+      <c r="K16" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L16" s="30" t="s">
+      <c r="L16" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M16" s="30"/>
-      <c r="N16" s="30">
+      <c r="M16" s="10"/>
+      <c r="N16" s="10">
         <v>10</v>
       </c>
-      <c r="O16" s="30">
+      <c r="O16" s="10">
         <v>10</v>
       </c>
-      <c r="P16" s="30">
+      <c r="P16" s="10">
         <v>36</v>
       </c>
-      <c r="Q16" s="30" t="s">
+      <c r="Q16" s="10" t="s">
         <v>144</v>
       </c>
-      <c r="R16" s="30" t="s">
+      <c r="R16" s="10" t="s">
         <v>145</v>
       </c>
-      <c r="S16" s="30">
+      <c r="S16" s="10">
         <v>25643429</v>
       </c>
-      <c r="T16" s="30" t="s">
+      <c r="T16" s="10" t="s">
         <v>146</v>
       </c>
-      <c r="U16" s="27" t="s">
+      <c r="U16" s="7" t="s">
         <v>147</v>
       </c>
-      <c r="V16" s="28" t="s">
+      <c r="V16" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W16" s="35"/>
-      <c r="X16" s="35"/>
-      <c r="Y16" s="35"/>
+      <c r="W16" s="15"/>
+      <c r="X16" s="15"/>
+      <c r="Y16" s="15"/>
     </row>
     <row r="17" spans="1:25" ht="30" customHeight="1">
-      <c r="A17" s="30">
+      <c r="A17" s="10">
         <v>7</v>
       </c>
-      <c r="B17" s="28">
+      <c r="B17" s="8">
         <v>11717129491</v>
       </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="30" t="s">
+      <c r="C17" s="8"/>
+      <c r="D17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="E17" s="30" t="s">
+      <c r="E17" s="10" t="s">
         <v>49</v>
       </c>
-      <c r="F17" s="30" t="s">
+      <c r="F17" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G17" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H17" s="30">
+      <c r="G17" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H17" s="10">
         <v>10</v>
       </c>
-      <c r="I17" s="31">
+      <c r="I17" s="11">
         <v>11</v>
       </c>
-      <c r="J17" s="31">
+      <c r="J17" s="11">
         <v>2017</v>
       </c>
-      <c r="K17" s="38" t="s">
+      <c r="K17" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L17" s="30" t="s">
+      <c r="L17" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M17" s="30"/>
-      <c r="N17" s="30">
+      <c r="M17" s="10"/>
+      <c r="N17" s="10">
         <v>8</v>
       </c>
-      <c r="O17" s="30">
+      <c r="O17" s="10">
         <v>8</v>
       </c>
-      <c r="P17" s="30">
+      <c r="P17" s="10">
         <v>36</v>
       </c>
-      <c r="Q17" s="30" t="s">
+      <c r="Q17" s="10" t="s">
         <v>48</v>
       </c>
-      <c r="R17" s="30" t="s">
+      <c r="R17" s="10" t="s">
         <v>51</v>
       </c>
-      <c r="S17" s="30">
+      <c r="S17" s="10">
         <v>17129491</v>
       </c>
-      <c r="T17" s="30" t="s">
+      <c r="T17" s="10" t="s">
         <v>52</v>
       </c>
-      <c r="U17" s="32" t="s">
+      <c r="U17" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="V17" s="28" t="s">
+      <c r="V17" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W17" s="35"/>
-      <c r="X17" s="35"/>
-      <c r="Y17" s="35"/>
+      <c r="W17" s="15"/>
+      <c r="X17" s="15"/>
+      <c r="Y17" s="15"/>
     </row>
     <row r="18" spans="1:25" ht="31.5">
-      <c r="A18" s="30">
+      <c r="A18" s="10">
         <v>8</v>
       </c>
-      <c r="B18" s="30">
+      <c r="B18" s="10">
         <v>11717864948</v>
       </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="30" t="s">
+      <c r="C18" s="10"/>
+      <c r="D18" s="10" t="s">
         <v>55</v>
       </c>
-      <c r="E18" s="30" t="s">
+      <c r="E18" s="10" t="s">
         <v>56</v>
       </c>
-      <c r="F18" s="30" t="s">
+      <c r="F18" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G18" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H18" s="30">
+      <c r="G18" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H18" s="10">
         <v>26</v>
       </c>
-      <c r="I18" s="31">
+      <c r="I18" s="11">
         <v>10</v>
       </c>
-      <c r="J18" s="31">
+      <c r="J18" s="11">
         <v>2017</v>
       </c>
-      <c r="K18" s="38" t="s">
+      <c r="K18" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L18" s="30" t="s">
+      <c r="L18" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M18" s="30"/>
-      <c r="N18" s="30">
+      <c r="M18" s="10"/>
+      <c r="N18" s="10">
         <v>10</v>
       </c>
-      <c r="O18" s="30">
+      <c r="O18" s="10">
         <v>10</v>
       </c>
-      <c r="P18" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q18" s="30" t="s">
+      <c r="P18" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q18" s="10" t="s">
         <v>58</v>
       </c>
-      <c r="R18" s="30" t="s">
+      <c r="R18" s="10" t="s">
         <v>59</v>
       </c>
-      <c r="S18" s="30">
+      <c r="S18" s="10">
         <v>17864948</v>
       </c>
-      <c r="T18" s="30" t="s">
+      <c r="T18" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="U18" s="32" t="s">
+      <c r="U18" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="V18" s="28" t="s">
+      <c r="V18" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W18" s="35"/>
-      <c r="X18" s="35"/>
-      <c r="Y18" s="35"/>
+      <c r="W18" s="15"/>
+      <c r="X18" s="15"/>
+      <c r="Y18" s="15"/>
     </row>
     <row r="19" spans="1:25" ht="15.75">
-      <c r="A19" s="30">
+      <c r="A19" s="10">
         <v>9</v>
       </c>
-      <c r="B19" s="30">
+      <c r="B19" s="10">
         <v>11717894774</v>
       </c>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30" t="s">
+      <c r="C19" s="10"/>
+      <c r="D19" s="10" t="s">
         <v>62</v>
       </c>
-      <c r="E19" s="30" t="s">
+      <c r="E19" s="10" t="s">
         <v>63</v>
       </c>
-      <c r="F19" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G19" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H19" s="30">
+      <c r="F19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G19" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H19" s="10">
         <v>12</v>
       </c>
-      <c r="I19" s="31">
+      <c r="I19" s="11">
         <v>12</v>
       </c>
-      <c r="J19" s="31">
+      <c r="J19" s="11">
         <v>2017</v>
       </c>
-      <c r="K19" s="38" t="s">
+      <c r="K19" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L19" s="30" t="s">
+      <c r="L19" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M19" s="30"/>
-      <c r="N19" s="30">
+      <c r="M19" s="10"/>
+      <c r="N19" s="10">
         <v>8</v>
       </c>
-      <c r="O19" s="30">
+      <c r="O19" s="10">
         <v>8</v>
       </c>
-      <c r="P19" s="30">
+      <c r="P19" s="10">
         <v>33</v>
       </c>
-      <c r="Q19" s="30" t="s">
+      <c r="Q19" s="10" t="s">
         <v>64</v>
       </c>
-      <c r="R19" s="30" t="s">
+      <c r="R19" s="10" t="s">
         <v>65</v>
       </c>
-      <c r="S19" s="30">
+      <c r="S19" s="10">
         <v>17894774</v>
       </c>
-      <c r="T19" s="30" t="s">
+      <c r="T19" s="10" t="s">
         <v>66</v>
       </c>
-      <c r="U19" s="32" t="s">
+      <c r="U19" s="12" t="s">
         <v>67</v>
       </c>
-      <c r="V19" s="28" t="s">
+      <c r="V19" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W19" s="35"/>
-      <c r="X19" s="35"/>
-      <c r="Y19" s="35"/>
+      <c r="W19" s="15"/>
+      <c r="X19" s="15"/>
+      <c r="Y19" s="15"/>
     </row>
     <row r="20" spans="1:25" ht="15.75">
-      <c r="A20" s="30">
+      <c r="A20" s="10">
         <v>10</v>
       </c>
-      <c r="B20" s="30">
+      <c r="B20" s="10">
         <v>11718797834</v>
       </c>
-      <c r="C20" s="30"/>
-      <c r="D20" s="30" t="s">
+      <c r="C20" s="10"/>
+      <c r="D20" s="10" t="s">
         <v>68</v>
       </c>
-      <c r="E20" s="30" t="s">
+      <c r="E20" s="10" t="s">
         <v>69</v>
       </c>
-      <c r="F20" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G20" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H20" s="30">
+      <c r="F20" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G20" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H20" s="10">
         <v>12</v>
       </c>
-      <c r="I20" s="31">
+      <c r="I20" s="11">
         <v>10</v>
       </c>
-      <c r="J20" s="31">
+      <c r="J20" s="11">
         <v>2017</v>
       </c>
-      <c r="K20" s="30" t="s">
+      <c r="K20" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L20" s="30" t="s">
+      <c r="L20" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M20" s="30"/>
-      <c r="N20" s="30">
+      <c r="M20" s="10"/>
+      <c r="N20" s="10">
         <v>8</v>
       </c>
-      <c r="O20" s="30">
+      <c r="O20" s="10">
         <v>8</v>
       </c>
-      <c r="P20" s="30">
+      <c r="P20" s="10">
         <v>34</v>
       </c>
-      <c r="Q20" s="30" t="s">
+      <c r="Q20" s="10" t="s">
         <v>71</v>
       </c>
-      <c r="R20" s="30" t="s">
+      <c r="R20" s="10" t="s">
         <v>72</v>
       </c>
-      <c r="S20" s="30">
+      <c r="S20" s="10">
         <v>17864948</v>
       </c>
-      <c r="T20" s="30" t="s">
+      <c r="T20" s="10" t="s">
         <v>60</v>
       </c>
-      <c r="U20" s="32" t="s">
+      <c r="U20" s="12" t="s">
         <v>53</v>
       </c>
-      <c r="V20" s="28" t="s">
+      <c r="V20" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W20" s="35"/>
-      <c r="X20" s="35"/>
-      <c r="Y20" s="35"/>
+      <c r="W20" s="15"/>
+      <c r="X20" s="15"/>
+      <c r="Y20" s="15"/>
     </row>
     <row r="21" spans="1:25" ht="31.5">
-      <c r="A21" s="30">
+      <c r="A21" s="10">
         <v>11</v>
       </c>
-      <c r="B21" s="30">
+      <c r="B21" s="10">
         <v>11719071798</v>
       </c>
-      <c r="C21" s="30"/>
-      <c r="D21" s="30" t="s">
+      <c r="C21" s="10"/>
+      <c r="D21" s="10" t="s">
         <v>75</v>
       </c>
-      <c r="E21" s="30" t="s">
+      <c r="E21" s="10" t="s">
         <v>76</v>
       </c>
-      <c r="F21" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G21" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H21" s="30">
+      <c r="F21" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H21" s="10">
         <v>18</v>
       </c>
-      <c r="I21" s="31">
+      <c r="I21" s="11">
         <v>5</v>
       </c>
-      <c r="J21" s="31">
+      <c r="J21" s="11">
         <v>2017</v>
       </c>
-      <c r="K21" s="30" t="s">
+      <c r="K21" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L21" s="30" t="s">
+      <c r="L21" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M21" s="30"/>
-      <c r="N21" s="30">
+      <c r="M21" s="10"/>
+      <c r="N21" s="10">
         <v>8</v>
       </c>
-      <c r="O21" s="30">
+      <c r="O21" s="10">
         <v>8</v>
       </c>
-      <c r="P21" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q21" s="30" t="s">
+      <c r="P21" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q21" s="10" t="s">
         <v>73</v>
       </c>
-      <c r="R21" s="30" t="s">
+      <c r="R21" s="10" t="s">
         <v>74</v>
       </c>
-      <c r="S21" s="30">
+      <c r="S21" s="10">
         <v>19071798</v>
       </c>
-      <c r="T21" s="30" t="s">
+      <c r="T21" s="10" t="s">
         <v>77</v>
       </c>
-      <c r="U21" s="32" t="s">
+      <c r="U21" s="12" t="s">
         <v>78</v>
       </c>
-      <c r="V21" s="28" t="s">
+      <c r="V21" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W21" s="35"/>
-      <c r="X21" s="35"/>
-      <c r="Y21" s="35"/>
+      <c r="W21" s="15"/>
+      <c r="X21" s="15"/>
+      <c r="Y21" s="15"/>
     </row>
     <row r="22" spans="1:25" ht="31.5">
-      <c r="A22" s="30">
+      <c r="A22" s="10">
         <v>12</v>
       </c>
-      <c r="B22" s="30">
+      <c r="B22" s="10">
         <v>11720010470</v>
       </c>
-      <c r="C22" s="30"/>
-      <c r="D22" s="30" t="s">
+      <c r="C22" s="10"/>
+      <c r="D22" s="10" t="s">
         <v>98</v>
       </c>
-      <c r="E22" s="30" t="s">
+      <c r="E22" s="10" t="s">
         <v>99</v>
       </c>
-      <c r="F22" s="30" t="s">
+      <c r="F22" s="10" t="s">
         <v>100</v>
       </c>
-      <c r="G22" s="30" t="s">
+      <c r="G22" s="10" t="s">
         <v>101</v>
       </c>
-      <c r="H22" s="30">
+      <c r="H22" s="10">
         <v>7</v>
       </c>
-      <c r="I22" s="31">
+      <c r="I22" s="11">
         <v>8</v>
       </c>
-      <c r="J22" s="31">
+      <c r="J22" s="11">
         <v>2017</v>
       </c>
-      <c r="K22" s="30" t="s">
+      <c r="K22" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L22" s="30" t="s">
+      <c r="L22" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M22" s="30"/>
-      <c r="N22" s="30">
+      <c r="M22" s="10"/>
+      <c r="N22" s="10">
         <v>10</v>
       </c>
-      <c r="O22" s="30">
+      <c r="O22" s="10">
         <v>10</v>
       </c>
-      <c r="P22" s="30">
+      <c r="P22" s="10">
         <v>36</v>
       </c>
-      <c r="Q22" s="30" t="s">
+      <c r="Q22" s="10" t="s">
         <v>102</v>
       </c>
-      <c r="R22" s="30" t="s">
+      <c r="R22" s="10" t="s">
         <v>103</v>
       </c>
-      <c r="S22" s="30">
+      <c r="S22" s="10">
         <v>20010470</v>
       </c>
-      <c r="T22" s="30" t="s">
+      <c r="T22" s="10" t="s">
         <v>104</v>
       </c>
-      <c r="U22" s="32" t="s">
+      <c r="U22" s="12" t="s">
         <v>105</v>
       </c>
-      <c r="V22" s="28" t="s">
+      <c r="V22" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W22" s="35"/>
-      <c r="X22" s="35"/>
-      <c r="Y22" s="35"/>
+      <c r="W22" s="15"/>
+      <c r="X22" s="15"/>
+      <c r="Y22" s="15"/>
     </row>
     <row r="23" spans="1:25" ht="31.5">
-      <c r="A23" s="30">
+      <c r="A23" s="10">
         <v>13</v>
       </c>
-      <c r="B23" s="30">
+      <c r="B23" s="10">
         <v>11720118025</v>
       </c>
-      <c r="C23" s="30"/>
-      <c r="D23" s="30" t="s">
+      <c r="C23" s="10"/>
+      <c r="D23" s="10" t="s">
         <v>92</v>
       </c>
-      <c r="E23" s="30" t="s">
+      <c r="E23" s="10" t="s">
         <v>93</v>
       </c>
-      <c r="F23" s="30" t="s">
+      <c r="F23" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G23" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H23" s="30">
+      <c r="G23" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H23" s="10">
         <v>28</v>
       </c>
-      <c r="I23" s="31">
+      <c r="I23" s="11">
         <v>2</v>
       </c>
-      <c r="J23" s="31">
+      <c r="J23" s="11">
         <v>2017</v>
       </c>
-      <c r="K23" s="30" t="s">
+      <c r="K23" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L23" s="30" t="s">
+      <c r="L23" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M23" s="30"/>
-      <c r="N23" s="30">
+      <c r="M23" s="10"/>
+      <c r="N23" s="10">
         <v>10</v>
       </c>
-      <c r="O23" s="30">
+      <c r="O23" s="10">
         <v>10</v>
       </c>
-      <c r="P23" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q23" s="30" t="s">
+      <c r="P23" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q23" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="R23" s="30" t="s">
+      <c r="R23" s="10" t="s">
         <v>95</v>
       </c>
-      <c r="S23" s="30">
+      <c r="S23" s="10">
         <v>20118025</v>
       </c>
-      <c r="T23" s="30" t="s">
+      <c r="T23" s="10" t="s">
         <v>96</v>
       </c>
-      <c r="U23" s="32" t="s">
+      <c r="U23" s="12" t="s">
         <v>97</v>
       </c>
-      <c r="V23" s="28" t="s">
+      <c r="V23" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W23" s="35"/>
-      <c r="X23" s="35"/>
-      <c r="Y23" s="35"/>
+      <c r="W23" s="15"/>
+      <c r="X23" s="15"/>
+      <c r="Y23" s="15"/>
     </row>
     <row r="24" spans="1:25" ht="15.75">
-      <c r="A24" s="30">
+      <c r="A24" s="10">
         <v>14</v>
       </c>
-      <c r="B24" s="30">
+      <c r="B24" s="10">
         <v>11720832435</v>
       </c>
-      <c r="C24" s="30"/>
-      <c r="D24" s="30" t="s">
+      <c r="C24" s="10"/>
+      <c r="D24" s="10" t="s">
         <v>79</v>
       </c>
-      <c r="E24" s="33" t="s">
+      <c r="E24" s="13" t="s">
         <v>80</v>
       </c>
-      <c r="F24" s="30" t="s">
+      <c r="F24" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G24" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H24" s="30">
+      <c r="G24" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H24" s="10">
         <v>10</v>
       </c>
-      <c r="I24" s="31">
+      <c r="I24" s="11">
         <v>11</v>
       </c>
-      <c r="J24" s="31">
+      <c r="J24" s="11">
         <v>2017</v>
       </c>
-      <c r="K24" s="38" t="s">
+      <c r="K24" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L24" s="30" t="s">
+      <c r="L24" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M24" s="30"/>
-      <c r="N24" s="30">
+      <c r="M24" s="10"/>
+      <c r="N24" s="10">
         <v>8</v>
       </c>
-      <c r="O24" s="30">
+      <c r="O24" s="10">
         <v>8</v>
       </c>
-      <c r="P24" s="30">
+      <c r="P24" s="10">
         <v>34</v>
       </c>
-      <c r="Q24" s="30" t="s">
+      <c r="Q24" s="10" t="s">
         <v>82</v>
       </c>
-      <c r="R24" s="30" t="s">
+      <c r="R24" s="10" t="s">
         <v>83</v>
       </c>
-      <c r="S24" s="30">
+      <c r="S24" s="10">
         <v>20832435</v>
       </c>
-      <c r="T24" s="30" t="s">
+      <c r="T24" s="10" t="s">
         <v>84</v>
       </c>
-      <c r="U24" s="32" t="s">
+      <c r="U24" s="12" t="s">
         <v>85</v>
       </c>
-      <c r="V24" s="28" t="s">
+      <c r="V24" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W24" s="35"/>
-      <c r="X24" s="35"/>
-      <c r="Y24" s="35"/>
+      <c r="W24" s="15"/>
+      <c r="X24" s="15"/>
+      <c r="Y24" s="15"/>
     </row>
     <row r="25" spans="1:25" ht="30" customHeight="1">
-      <c r="A25" s="30">
+      <c r="A25" s="10">
         <v>16</v>
       </c>
-      <c r="B25" s="30">
+      <c r="B25" s="10">
         <v>11722655443</v>
       </c>
-      <c r="C25" s="30"/>
-      <c r="D25" s="30" t="s">
+      <c r="C25" s="10"/>
+      <c r="D25" s="10" t="s">
         <v>94</v>
       </c>
-      <c r="E25" s="30" t="s">
+      <c r="E25" s="10" t="s">
         <v>112</v>
       </c>
-      <c r="F25" s="30" t="s">
+      <c r="F25" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G25" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H25" s="30">
+      <c r="G25" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H25" s="10">
         <v>18</v>
       </c>
-      <c r="I25" s="31">
+      <c r="I25" s="11">
         <v>11</v>
       </c>
-      <c r="J25" s="31">
+      <c r="J25" s="11">
         <v>2017</v>
       </c>
-      <c r="K25" s="38" t="s">
+      <c r="K25" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L25" s="30" t="s">
+      <c r="L25" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M25" s="30"/>
-      <c r="N25" s="30">
+      <c r="M25" s="10"/>
+      <c r="N25" s="10">
         <v>10</v>
       </c>
-      <c r="O25" s="30">
+      <c r="O25" s="10">
         <v>10</v>
       </c>
-      <c r="P25" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q25" s="30" t="s">
+      <c r="P25" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q25" s="10" t="s">
         <v>44</v>
       </c>
-      <c r="R25" s="30" t="s">
+      <c r="R25" s="10" t="s">
         <v>113</v>
       </c>
-      <c r="S25" s="30">
+      <c r="S25" s="10">
         <v>9475732</v>
       </c>
-      <c r="T25" s="30" t="s">
+      <c r="T25" s="10" t="s">
         <v>114</v>
       </c>
-      <c r="U25" s="32" t="s">
+      <c r="U25" s="12" t="s">
         <v>115</v>
       </c>
-      <c r="V25" s="28" t="s">
+      <c r="V25" s="8" t="s">
         <v>116</v>
       </c>
-      <c r="W25" s="35"/>
-      <c r="X25" s="35"/>
-      <c r="Y25" s="35"/>
+      <c r="W25" s="15"/>
+      <c r="X25" s="15"/>
+      <c r="Y25" s="15"/>
     </row>
     <row r="26" spans="1:25" ht="15.75">
-      <c r="A26" s="30">
+      <c r="A26" s="10">
         <v>17</v>
       </c>
-      <c r="B26" s="30">
+      <c r="B26" s="10">
         <v>11722655654</v>
       </c>
-      <c r="C26" s="30"/>
-      <c r="D26" s="30" t="s">
+      <c r="C26" s="10"/>
+      <c r="D26" s="10" t="s">
         <v>117</v>
       </c>
-      <c r="E26" s="30" t="s">
+      <c r="E26" s="10" t="s">
         <v>118</v>
       </c>
-      <c r="F26" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G26" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H26" s="30">
+      <c r="F26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G26" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H26" s="10">
         <v>17</v>
       </c>
-      <c r="I26" s="31">
+      <c r="I26" s="11">
         <v>8</v>
       </c>
-      <c r="J26" s="31">
+      <c r="J26" s="11">
         <v>2017</v>
       </c>
-      <c r="K26" s="38" t="s">
+      <c r="K26" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L26" s="30" t="s">
+      <c r="L26" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M26" s="30"/>
-      <c r="N26" s="30">
+      <c r="M26" s="10"/>
+      <c r="N26" s="10">
         <v>10</v>
       </c>
-      <c r="O26" s="30">
+      <c r="O26" s="10">
         <v>10</v>
       </c>
-      <c r="P26" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q26" s="30" t="s">
+      <c r="P26" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q26" s="10" t="s">
         <v>119</v>
       </c>
-      <c r="R26" s="30" t="s">
+      <c r="R26" s="10" t="s">
         <v>120</v>
       </c>
-      <c r="S26" s="30">
+      <c r="S26" s="10">
         <v>22655654</v>
       </c>
-      <c r="T26" s="30" t="s">
+      <c r="T26" s="10" t="s">
         <v>121</v>
       </c>
-      <c r="U26" s="32" t="s">
+      <c r="U26" s="12" t="s">
         <v>122</v>
       </c>
-      <c r="V26" s="28" t="s">
+      <c r="V26" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W26" s="35"/>
-      <c r="X26" s="35"/>
-      <c r="Y26" s="35"/>
+      <c r="W26" s="15"/>
+      <c r="X26" s="15"/>
+      <c r="Y26" s="15"/>
     </row>
     <row r="27" spans="1:25" ht="15.75">
-      <c r="A27" s="30">
+      <c r="A27" s="10">
         <v>18</v>
       </c>
-      <c r="B27" s="30">
+      <c r="B27" s="10">
         <v>11725150838</v>
       </c>
-      <c r="C27" s="30"/>
-      <c r="D27" s="30" t="s">
+      <c r="C27" s="10"/>
+      <c r="D27" s="10" t="s">
         <v>130</v>
       </c>
-      <c r="E27" s="30" t="s">
+      <c r="E27" s="10" t="s">
         <v>131</v>
       </c>
-      <c r="F27" s="30" t="s">
+      <c r="F27" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G27" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H27" s="30">
+      <c r="G27" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H27" s="10">
         <v>26</v>
       </c>
-      <c r="I27" s="31">
+      <c r="I27" s="11">
         <v>12</v>
       </c>
-      <c r="J27" s="31">
+      <c r="J27" s="11">
         <v>2017</v>
       </c>
-      <c r="K27" s="30" t="s">
+      <c r="K27" s="10" t="s">
         <v>70</v>
       </c>
-      <c r="L27" s="30" t="s">
+      <c r="L27" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M27" s="30"/>
-      <c r="N27" s="30">
+      <c r="M27" s="10"/>
+      <c r="N27" s="10">
         <v>10</v>
       </c>
-      <c r="O27" s="30">
+      <c r="O27" s="10">
         <v>10</v>
       </c>
-      <c r="P27" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q27" s="30" t="s">
+      <c r="P27" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q27" s="10" t="s">
         <v>132</v>
       </c>
-      <c r="R27" s="30" t="s">
+      <c r="R27" s="10" t="s">
         <v>133</v>
       </c>
-      <c r="S27" s="30">
+      <c r="S27" s="10">
         <v>25150838</v>
       </c>
-      <c r="T27" s="30" t="s">
+      <c r="T27" s="10" t="s">
         <v>134</v>
       </c>
-      <c r="U27" s="32" t="s">
+      <c r="U27" s="12" t="s">
         <v>135</v>
       </c>
-      <c r="V27" s="28" t="s">
+      <c r="V27" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W27" s="35"/>
-      <c r="X27" s="35"/>
-      <c r="Y27" s="35"/>
+      <c r="W27" s="15"/>
+      <c r="X27" s="15"/>
+      <c r="Y27" s="15"/>
     </row>
     <row r="28" spans="1:25" ht="31.5">
-      <c r="A28" s="30">
+      <c r="A28" s="10">
         <v>19</v>
       </c>
-      <c r="B28" s="30">
+      <c r="B28" s="10">
         <v>11725643421</v>
       </c>
-      <c r="C28" s="30"/>
-      <c r="D28" s="30" t="s">
+      <c r="C28" s="10"/>
+      <c r="D28" s="10" t="s">
         <v>136</v>
       </c>
-      <c r="E28" s="30" t="s">
+      <c r="E28" s="10" t="s">
         <v>137</v>
       </c>
-      <c r="F28" s="30" t="s">
+      <c r="F28" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G28" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H28" s="30">
+      <c r="G28" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H28" s="10">
         <v>4</v>
       </c>
-      <c r="I28" s="31">
+      <c r="I28" s="11">
         <v>12</v>
       </c>
-      <c r="J28" s="31">
+      <c r="J28" s="11">
         <v>2017</v>
       </c>
-      <c r="K28" s="38" t="s">
+      <c r="K28" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L28" s="30" t="s">
+      <c r="L28" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M28" s="30"/>
-      <c r="N28" s="30">
+      <c r="M28" s="10"/>
+      <c r="N28" s="10">
         <v>8</v>
       </c>
-      <c r="O28" s="30">
+      <c r="O28" s="10">
         <v>8</v>
       </c>
-      <c r="P28" s="30">
+      <c r="P28" s="10">
         <v>34</v>
       </c>
-      <c r="Q28" s="30" t="s">
+      <c r="Q28" s="10" t="s">
         <v>138</v>
       </c>
-      <c r="R28" s="30" t="s">
+      <c r="R28" s="10" t="s">
         <v>139</v>
       </c>
-      <c r="S28" s="30">
+      <c r="S28" s="10">
         <v>25643421</v>
       </c>
-      <c r="T28" s="30" t="s">
+      <c r="T28" s="10" t="s">
         <v>140</v>
       </c>
-      <c r="U28" s="32" t="s">
+      <c r="U28" s="12" t="s">
         <v>141</v>
       </c>
-      <c r="V28" s="28" t="s">
+      <c r="V28" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W28" s="35"/>
-      <c r="X28" s="35"/>
-      <c r="Y28" s="35"/>
+      <c r="W28" s="15"/>
+      <c r="X28" s="15"/>
+      <c r="Y28" s="15"/>
     </row>
     <row r="29" spans="1:25" ht="30" customHeight="1">
-      <c r="A29" s="30">
+      <c r="A29" s="10">
         <v>20</v>
       </c>
-      <c r="B29" s="28">
+      <c r="B29" s="8">
         <v>11814699917</v>
       </c>
-      <c r="C29" s="28"/>
-      <c r="D29" s="30" t="s">
+      <c r="C29" s="8"/>
+      <c r="D29" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="E29" s="30" t="s">
+      <c r="E29" s="10" t="s">
         <v>39</v>
       </c>
-      <c r="F29" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G29" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H29" s="30">
+      <c r="F29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G29" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H29" s="10">
         <v>5</v>
       </c>
-      <c r="I29" s="31">
+      <c r="I29" s="11">
         <v>1</v>
       </c>
-      <c r="J29" s="31">
+      <c r="J29" s="11">
         <v>2017</v>
       </c>
-      <c r="K29" s="38" t="s">
+      <c r="K29" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L29" s="30" t="s">
+      <c r="L29" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M29" s="30"/>
-      <c r="N29" s="30">
+      <c r="M29" s="10"/>
+      <c r="N29" s="10">
         <v>8</v>
       </c>
-      <c r="O29" s="30">
+      <c r="O29" s="10">
         <v>8</v>
       </c>
-      <c r="P29" s="30">
+      <c r="P29" s="10">
         <v>34</v>
       </c>
-      <c r="Q29" s="30" t="s">
+      <c r="Q29" s="10" t="s">
         <v>40</v>
       </c>
-      <c r="R29" s="30" t="s">
+      <c r="R29" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="S29" s="28">
+      <c r="S29" s="8">
         <v>14699917</v>
       </c>
-      <c r="T29" s="28" t="s">
+      <c r="T29" s="8" t="s">
         <v>32</v>
       </c>
-      <c r="U29" s="28" t="s">
+      <c r="U29" s="8" t="s">
         <v>33</v>
       </c>
-      <c r="V29" s="28" t="s">
+      <c r="V29" s="8" t="s">
         <v>31</v>
       </c>
-      <c r="W29" s="35"/>
-      <c r="X29" s="35"/>
-      <c r="Y29" s="35"/>
+      <c r="W29" s="15"/>
+      <c r="X29" s="15"/>
+      <c r="Y29" s="15"/>
     </row>
     <row r="30" spans="1:25" ht="15.75">
-      <c r="A30" s="28">
+      <c r="A30" s="8">
         <v>21</v>
       </c>
-      <c r="B30" s="30">
+      <c r="B30" s="10">
         <v>11820435077</v>
       </c>
-      <c r="C30" s="30"/>
-      <c r="D30" s="30" t="s">
+      <c r="C30" s="10"/>
+      <c r="D30" s="10" t="s">
         <v>86</v>
       </c>
-      <c r="E30" s="30" t="s">
+      <c r="E30" s="10" t="s">
         <v>87</v>
       </c>
-      <c r="F30" s="30" t="s">
+      <c r="F30" s="10" t="s">
         <v>57</v>
       </c>
-      <c r="G30" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H30" s="30">
+      <c r="G30" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H30" s="10">
         <v>26</v>
       </c>
-      <c r="I30" s="31">
+      <c r="I30" s="11">
         <v>1</v>
       </c>
-      <c r="J30" s="31">
+      <c r="J30" s="11">
         <v>2018</v>
       </c>
-      <c r="K30" s="38" t="s">
+      <c r="K30" s="18" t="s">
         <v>27</v>
       </c>
-      <c r="L30" s="30" t="s">
+      <c r="L30" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M30" s="30"/>
-      <c r="N30" s="30">
+      <c r="M30" s="10"/>
+      <c r="N30" s="10">
         <v>8</v>
       </c>
-      <c r="O30" s="30">
+      <c r="O30" s="10">
         <v>8</v>
       </c>
-      <c r="P30" s="30">
+      <c r="P30" s="10">
         <v>34</v>
       </c>
-      <c r="Q30" s="30" t="s">
+      <c r="Q30" s="10" t="s">
         <v>88</v>
       </c>
-      <c r="R30" s="33" t="s">
+      <c r="R30" s="13" t="s">
         <v>89</v>
       </c>
-      <c r="S30" s="30">
+      <c r="S30" s="10">
         <v>20435077</v>
       </c>
-      <c r="T30" s="30" t="s">
+      <c r="T30" s="10" t="s">
         <v>90</v>
       </c>
-      <c r="U30" s="32" t="s">
+      <c r="U30" s="12" t="s">
         <v>91</v>
       </c>
-      <c r="V30" s="28" t="s">
+      <c r="V30" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W30" s="35"/>
-      <c r="X30" s="35"/>
-      <c r="Y30" s="35"/>
+      <c r="W30" s="15"/>
+      <c r="X30" s="15"/>
+      <c r="Y30" s="15"/>
     </row>
     <row r="31" spans="1:25" ht="15.75" customHeight="1">
-      <c r="A31" s="36">
+      <c r="A31" s="16">
         <v>22</v>
       </c>
-      <c r="B31" s="29">
+      <c r="B31" s="9">
         <v>11313966325</v>
       </c>
-      <c r="C31" s="30"/>
-      <c r="D31" s="30" t="s">
+      <c r="C31" s="10"/>
+      <c r="D31" s="10" t="s">
         <v>34</v>
       </c>
-      <c r="E31" s="30" t="s">
+      <c r="E31" s="10" t="s">
         <v>50</v>
       </c>
-      <c r="F31" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="G31" s="30" t="s">
-        <v>35</v>
-      </c>
-      <c r="H31" s="30">
+      <c r="F31" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>35</v>
+      </c>
+      <c r="H31" s="10">
         <v>15</v>
       </c>
-      <c r="I31" s="31">
+      <c r="I31" s="11">
         <v>8</v>
       </c>
-      <c r="J31" s="31">
+      <c r="J31" s="11">
         <v>2017</v>
       </c>
-      <c r="K31" s="34" t="s">
+      <c r="K31" s="14" t="s">
         <v>27</v>
       </c>
-      <c r="L31" s="30" t="s">
+      <c r="L31" s="10" t="s">
         <v>28</v>
       </c>
-      <c r="M31" s="30"/>
-      <c r="N31" s="30">
+      <c r="M31" s="10"/>
+      <c r="N31" s="10">
         <v>8</v>
       </c>
-      <c r="O31" s="30">
+      <c r="O31" s="10">
         <v>8</v>
       </c>
-      <c r="P31" s="30">
-        <v>35</v>
-      </c>
-      <c r="Q31" s="30" t="s">
+      <c r="P31" s="10">
+        <v>35</v>
+      </c>
+      <c r="Q31" s="10" t="s">
         <v>36</v>
       </c>
-      <c r="R31" s="30" t="s">
+      <c r="R31" s="10" t="s">
         <v>37</v>
       </c>
-      <c r="S31" s="30">
+      <c r="S31" s="10">
         <v>13966325</v>
       </c>
-      <c r="T31" s="29" t="s">
+      <c r="T31" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="U31" s="29" t="s">
+      <c r="U31" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="V31" s="28" t="s">
+      <c r="V31" s="8" t="s">
         <v>54</v>
       </c>
-      <c r="W31" s="35"/>
-      <c r="X31" s="35"/>
-      <c r="Y31" s="35"/>
+      <c r="W31" s="15"/>
+      <c r="X31" s="15"/>
+      <c r="Y31" s="15"/>
     </row>
     <row r="32" spans="1:25" ht="15.75">
-      <c r="A32" s="35"/>
-      <c r="B32" s="35"/>
-      <c r="C32" s="35"/>
-      <c r="D32" s="35"/>
-      <c r="E32" s="35"/>
-      <c r="F32" s="35"/>
-      <c r="G32" s="35"/>
-      <c r="H32" s="35"/>
-      <c r="I32" s="35"/>
-      <c r="J32" s="35"/>
-      <c r="K32" s="35"/>
-      <c r="L32" s="35"/>
-      <c r="M32" s="35"/>
-      <c r="N32" s="35"/>
-      <c r="O32" s="35"/>
-      <c r="P32" s="35"/>
-      <c r="Q32" s="35"/>
-      <c r="R32" s="35"/>
-      <c r="S32" s="35"/>
-      <c r="T32" s="35"/>
-      <c r="U32" s="35"/>
-      <c r="V32" s="35"/>
-      <c r="W32" s="35"/>
-      <c r="X32" s="35"/>
-      <c r="Y32" s="35"/>
+      <c r="A32" s="15"/>
+      <c r="B32" s="15"/>
+      <c r="C32" s="15"/>
+      <c r="D32" s="15"/>
+      <c r="E32" s="15"/>
+      <c r="F32" s="15"/>
+      <c r="G32" s="15"/>
+      <c r="H32" s="15"/>
+      <c r="I32" s="15"/>
+      <c r="J32" s="15"/>
+      <c r="K32" s="15"/>
+      <c r="L32" s="15"/>
+      <c r="M32" s="15"/>
+      <c r="N32" s="15"/>
+      <c r="O32" s="15"/>
+      <c r="P32" s="15"/>
+      <c r="Q32" s="15"/>
+      <c r="R32" s="15"/>
+      <c r="S32" s="15"/>
+      <c r="T32" s="15"/>
+      <c r="U32" s="15"/>
+      <c r="V32" s="15"/>
+      <c r="W32" s="15"/>
+      <c r="X32" s="15"/>
+      <c r="Y32" s="15"/>
     </row>
     <row r="33" spans="1:25" ht="15.75">
-      <c r="A33" s="35"/>
-      <c r="B33" s="35"/>
-      <c r="C33" s="35"/>
-      <c r="D33" s="35"/>
-      <c r="E33" s="35"/>
-      <c r="F33" s="35"/>
-      <c r="G33" s="35"/>
-      <c r="H33" s="35"/>
-      <c r="I33" s="35"/>
-      <c r="J33" s="35"/>
-      <c r="K33" s="35"/>
-      <c r="L33" s="35"/>
-      <c r="M33" s="35"/>
-      <c r="N33" s="35"/>
-      <c r="O33" s="35"/>
-      <c r="P33" s="35"/>
-      <c r="Q33" s="35"/>
-      <c r="R33" s="35"/>
-      <c r="S33" s="35"/>
-      <c r="T33" s="35"/>
-      <c r="U33" s="35"/>
-      <c r="V33" s="35"/>
-      <c r="W33" s="35"/>
-      <c r="X33" s="35"/>
-      <c r="Y33" s="35"/>
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15"/>
+      <c r="D33" s="15"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15"/>
+      <c r="M33" s="15"/>
+      <c r="N33" s="15"/>
+      <c r="O33" s="15"/>
+      <c r="P33" s="15"/>
+      <c r="Q33" s="15"/>
+      <c r="R33" s="15"/>
+      <c r="S33" s="15"/>
+      <c r="T33" s="15"/>
+      <c r="U33" s="15"/>
+      <c r="V33" s="15"/>
+      <c r="W33" s="15"/>
+      <c r="X33" s="15"/>
+      <c r="Y33" s="15"/>
     </row>
     <row r="34" spans="1:25" ht="15.75">
-      <c r="A34" s="35"/>
-      <c r="B34" s="35"/>
-      <c r="C34" s="35"/>
-      <c r="D34" s="35"/>
-      <c r="E34" s="35"/>
-      <c r="F34" s="35"/>
-      <c r="G34" s="35"/>
-      <c r="H34" s="35"/>
-      <c r="I34" s="35"/>
-      <c r="J34" s="35"/>
-      <c r="K34" s="35"/>
-      <c r="L34" s="35"/>
-      <c r="M34" s="35"/>
-      <c r="N34" s="35"/>
-      <c r="O34" s="35"/>
-      <c r="P34" s="35"/>
-      <c r="Q34" s="35"/>
-      <c r="R34" s="35"/>
-      <c r="S34" s="35"/>
-      <c r="T34" s="35"/>
-      <c r="U34" s="35"/>
-      <c r="V34" s="35"/>
-      <c r="W34" s="35"/>
-      <c r="X34" s="35"/>
-      <c r="Y34" s="35"/>
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15"/>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15"/>
+      <c r="G34" s="15"/>
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+      <c r="O34" s="15"/>
+      <c r="P34" s="15"/>
+      <c r="Q34" s="15"/>
+      <c r="R34" s="15"/>
+      <c r="S34" s="15"/>
+      <c r="T34" s="15"/>
+      <c r="U34" s="15"/>
+      <c r="V34" s="15"/>
+      <c r="W34" s="15"/>
+      <c r="X34" s="15"/>
+      <c r="Y34" s="15"/>
     </row>
   </sheetData>
   <sortState ref="B11:V32">
     <sortCondition ref="B11"/>
   </sortState>
   <mergeCells count="40">
-    <mergeCell ref="V9:V10"/>
-    <mergeCell ref="S9:S10"/>
-    <mergeCell ref="T9:T10"/>
-    <mergeCell ref="U9:U10"/>
-    <mergeCell ref="Q9:R10"/>
-    <mergeCell ref="D9:E10"/>
-    <mergeCell ref="H9:J9"/>
-    <mergeCell ref="L9:M9"/>
-    <mergeCell ref="N9:P9"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="F9:F10"/>
-    <mergeCell ref="G9:G10"/>
-    <mergeCell ref="K9:K10"/>
-    <mergeCell ref="M7:N7"/>
-    <mergeCell ref="O7:R7"/>
-    <mergeCell ref="AB7:AD7"/>
-    <mergeCell ref="A8:P8"/>
-    <mergeCell ref="U7:V7"/>
-    <mergeCell ref="Q8:V8"/>
-    <mergeCell ref="A7:C7"/>
-    <mergeCell ref="D7:E7"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="H7:J7"/>
-    <mergeCell ref="K7:L7"/>
     <mergeCell ref="W5:X5"/>
     <mergeCell ref="Z5:AB5"/>
     <mergeCell ref="AD5:AE5"/>
@@ -3025,6 +3007,32 @@
     <mergeCell ref="AD6:AE6"/>
     <mergeCell ref="S6:V6"/>
     <mergeCell ref="A5:V5"/>
+    <mergeCell ref="M7:N7"/>
+    <mergeCell ref="O7:R7"/>
+    <mergeCell ref="AB7:AD7"/>
+    <mergeCell ref="A8:P8"/>
+    <mergeCell ref="U7:V7"/>
+    <mergeCell ref="Q8:V8"/>
+    <mergeCell ref="A7:C7"/>
+    <mergeCell ref="D7:E7"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="H7:J7"/>
+    <mergeCell ref="K7:L7"/>
+    <mergeCell ref="D9:E10"/>
+    <mergeCell ref="H9:J9"/>
+    <mergeCell ref="L9:M9"/>
+    <mergeCell ref="N9:P9"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="F9:F10"/>
+    <mergeCell ref="G9:G10"/>
+    <mergeCell ref="K9:K10"/>
+    <mergeCell ref="V9:V10"/>
+    <mergeCell ref="S9:S10"/>
+    <mergeCell ref="T9:T10"/>
+    <mergeCell ref="U9:U10"/>
+    <mergeCell ref="Q9:R10"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>